<commit_message>
Planilha reorganizada (preço sugerido ao lado do preço de hoje); obrigado com botões Excel e Google Planilhas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -140,7 +140,7 @@
     <t xml:space="preserve">Divulgação (anúncios, cartões, etc.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Reposição de equipamentos (lixa, alicate, lâmpada...)</t>
+    <t xml:space="preserve">Reposição de equipamentos (lixa, alicate)</t>
   </si>
   <si>
     <t xml:space="preserve">Média mensal</t>
@@ -212,7 +212,7 @@
     <t xml:space="preserve">Passo 2  ·  Preço sugerido por serviço</t>
   </si>
   <si>
-    <t xml:space="preserve">Células amarelas = você preenche. Os serviços abaixo são EXEMPLOS (valores ilustrativos): troque pelos seus.</t>
+    <t xml:space="preserve">Preencha as células amarelas (A a D). O PREÇO SUGERIDO aparece logo ao lado. Os serviços abaixo são EXEMPLOS: troque pelos seus.</t>
   </si>
   <si>
     <t xml:space="preserve">Serviço</t>
@@ -221,10 +221,16 @@
     <t xml:space="preserve">Tempo (min)</t>
   </si>
   <si>
-    <t xml:space="preserve">Material gasto (R$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preço que cobro hoje (R$)</t>
+    <t xml:space="preserve">Material (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobro hoje (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREÇO SUGERIDO (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Situação</t>
   </si>
   <si>
     <t xml:space="preserve">Custo do tempo (R$)</t>
@@ -233,15 +239,9 @@
     <t xml:space="preserve">Custo total (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">PREÇO SUGERIDO (R$)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lucro hoje (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Situação</t>
-  </si>
-  <si>
     <t xml:space="preserve">Esmaltação simples (mão)</t>
   </si>
   <si>
@@ -269,7 +269,7 @@
     <t xml:space="preserve">✦  Como o preço é calculado: (custo do tempo + material) ÷ (1 − taxa do cartão − margem), arredondado para cima ao real.</t>
   </si>
   <si>
-    <t xml:space="preserve">✦  Custo do tempo = minutos ÷ 60 × custo da sua hora (aba “Meu custo por hora”).</t>
+    <t xml:space="preserve">✦  Custo do tempo = minutos ÷ 60 × custo da sua hora (aba “Meu custo por hora”). As colunas de conta ficam à direita (G a I).</t>
   </si>
   <si>
     <t xml:space="preserve">✦  Lucro hoje = o que você cobra, menos a taxa do cartão, menos o custo total. Negativo = você paga para fazer esse serviço.</t>
@@ -857,7 +857,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1002,6 +1002,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="20" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1014,20 +1018,20 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="26" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="170" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1439,7 +1443,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Meus serviços'!$G$5:$G$14</c:f>
+              <c:f>'Meus serviços'!$E$5:$E$14</c:f>
               <c:numCache>
                 <c:formatCode>"R$ "#,##0.00</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1473,11 +1477,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="82976009"/>
-        <c:axId val="29108995"/>
+        <c:axId val="16946007"/>
+        <c:axId val="14740886"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="82976009"/>
+        <c:axId val="16946007"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1509,7 +1513,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29108995"/>
+        <c:crossAx val="14740886"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1517,7 +1521,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29108995"/>
+        <c:axId val="14740886"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1559,7 +1563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82976009"/>
+        <c:crossAx val="16946007"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2470,9 +2474,9 @@
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
   </cols>
   <sheetData>
@@ -2825,15 +2829,13 @@
   <dimension ref="A1:J37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
   </cols>
   <sheetData>
@@ -2890,758 +2892,758 @@
       <c r="D4" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="F4" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="35" t="s">
+      <c r="G4" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="34" t="s">
+      <c r="H4" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="I4" s="34" t="s">
+      <c r="I4" s="36" t="s">
         <v>71</v>
       </c>
       <c r="J4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="38" t="n">
         <v>45</v>
       </c>
-      <c r="C5" s="38" t="n">
+      <c r="C5" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="39" t="n">
         <v>35</v>
       </c>
-      <c r="E5" s="39" t="n">
+      <c r="E5" s="40" t="n">
+        <f aca="false">IF(B5="","",ROUNDUP(H5/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>36</v>
+      </c>
+      <c r="F5" s="41" t="str">
+        <f aca="false">IF(OR(B5="",D5=""),"",IF(D5&gt;=E5,"OK: cobre custos e margem",IF(I5&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>Atenção: pouca folga</v>
+      </c>
+      <c r="G5" s="42" t="n">
         <f aca="false">IF(B5="","",B5/60*'Meu custo por hora'!$B$25)</f>
         <v>26.7143364718422</v>
       </c>
-      <c r="F5" s="39" t="n">
-        <f aca="false">IF(B5="","",E5+C5)</f>
+      <c r="H5" s="42" t="n">
+        <f aca="false">IF(B5="","",G5+C5)</f>
         <v>30.7143364718422</v>
       </c>
-      <c r="G5" s="40" t="n">
-        <f aca="false">IF(B5="","",ROUNDUP(F5/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>36</v>
-      </c>
-      <c r="H5" s="41" t="n">
-        <f aca="false">IF(OR(B5="",D5=""),"",D5*(1-'Meu custo por hora'!$B$28)-F5)</f>
+      <c r="I5" s="43" t="n">
+        <f aca="false">IF(OR(B5="",D5=""),"",D5*(1-'Meu custo por hora'!$B$28)-H5)</f>
         <v>2.88566352815776</v>
       </c>
-      <c r="I5" s="42" t="str">
-        <f aca="false">IF(OR(B5="",D5=""),"",IF(D5&gt;=G5,"OK: preço cobre custos e margem",IF(H5&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>Atenção: pouca folga</v>
-      </c>
       <c r="J5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="38" t="n">
         <v>50</v>
       </c>
-      <c r="C6" s="38" t="n">
+      <c r="C6" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="38" t="n">
+      <c r="D6" s="39" t="n">
         <v>35</v>
       </c>
-      <c r="E6" s="39" t="n">
+      <c r="E6" s="40" t="n">
+        <f aca="false">IF(B6="","",ROUNDUP(H6/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>40</v>
+      </c>
+      <c r="F6" s="41" t="str">
+        <f aca="false">IF(OR(B6="",D6=""),"",IF(D6&gt;=E6,"OK: cobre custos e margem",IF(I6&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>PREJUÍZO: abaixo do custo</v>
+      </c>
+      <c r="G6" s="42" t="n">
         <f aca="false">IF(B6="","",B6/60*'Meu custo por hora'!$B$25)</f>
         <v>29.6825960798247</v>
       </c>
-      <c r="F6" s="39" t="n">
-        <f aca="false">IF(B6="","",E6+C6)</f>
+      <c r="H6" s="42" t="n">
+        <f aca="false">IF(B6="","",G6+C6)</f>
         <v>33.6825960798247</v>
       </c>
-      <c r="G6" s="40" t="n">
-        <f aca="false">IF(B6="","",ROUNDUP(F6/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>40</v>
-      </c>
-      <c r="H6" s="41" t="n">
-        <f aca="false">IF(OR(B6="",D6=""),"",D6*(1-'Meu custo por hora'!$B$28)-F6)</f>
+      <c r="I6" s="43" t="n">
+        <f aca="false">IF(OR(B6="",D6=""),"",D6*(1-'Meu custo por hora'!$B$28)-H6)</f>
         <v>-0.0825960798247181</v>
       </c>
-      <c r="I6" s="42" t="str">
-        <f aca="false">IF(OR(B6="",D6=""),"",IF(D6&gt;=G6,"OK: preço cobre custos e margem",IF(H6&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>PREJUÍZO: preço abaixo do custo</v>
-      </c>
       <c r="J6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="38" t="n">
         <v>90</v>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="39" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="E7" s="39" t="n">
+      <c r="E7" s="40" t="n">
+        <f aca="false">IF(B7="","",ROUNDUP(H7/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>72</v>
+      </c>
+      <c r="F7" s="41" t="str">
+        <f aca="false">IF(OR(B7="",D7=""),"",IF(D7&gt;=E7,"OK: cobre custos e margem",IF(I7&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>PREJUÍZO: abaixo do custo</v>
+      </c>
+      <c r="G7" s="42" t="n">
         <f aca="false">IF(B7="","",B7/60*'Meu custo por hora'!$B$25)</f>
         <v>53.4286729436845</v>
       </c>
-      <c r="F7" s="39" t="n">
-        <f aca="false">IF(B7="","",E7+C7)</f>
+      <c r="H7" s="42" t="n">
+        <f aca="false">IF(B7="","",G7+C7)</f>
         <v>61.4286729436845</v>
       </c>
-      <c r="G7" s="40" t="n">
-        <f aca="false">IF(B7="","",ROUNDUP(F7/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>72</v>
-      </c>
-      <c r="H7" s="41" t="n">
-        <f aca="false">IF(OR(B7="",D7=""),"",D7*(1-'Meu custo por hora'!$B$28)-F7)</f>
+      <c r="I7" s="43" t="n">
+        <f aca="false">IF(OR(B7="",D7=""),"",D7*(1-'Meu custo por hora'!$B$28)-H7)</f>
         <v>-3.8286729436845</v>
       </c>
-      <c r="I7" s="42" t="str">
-        <f aca="false">IF(OR(B7="",D7=""),"",IF(D7&gt;=G7,"OK: preço cobre custos e margem",IF(H7&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>PREJUÍZO: preço abaixo do custo</v>
-      </c>
       <c r="J7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="B8" s="38" t="n">
         <v>75</v>
       </c>
-      <c r="C8" s="38" t="n">
+      <c r="C8" s="39" t="n">
         <v>12</v>
       </c>
-      <c r="D8" s="38" t="n">
+      <c r="D8" s="39" t="n">
         <v>70</v>
       </c>
-      <c r="E8" s="39" t="n">
+      <c r="E8" s="40" t="n">
+        <f aca="false">IF(B8="","",ROUNDUP(H8/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>66</v>
+      </c>
+      <c r="F8" s="41" t="str">
+        <f aca="false">IF(OR(B8="",D8=""),"",IF(D8&gt;=E8,"OK: cobre custos e margem",IF(I8&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>OK: cobre custos e margem</v>
+      </c>
+      <c r="G8" s="42" t="n">
         <f aca="false">IF(B8="","",B8/60*'Meu custo por hora'!$B$25)</f>
         <v>44.5238941197371</v>
       </c>
-      <c r="F8" s="39" t="n">
-        <f aca="false">IF(B8="","",E8+C8)</f>
+      <c r="H8" s="42" t="n">
+        <f aca="false">IF(B8="","",G8+C8)</f>
         <v>56.5238941197371</v>
       </c>
-      <c r="G8" s="40" t="n">
-        <f aca="false">IF(B8="","",ROUNDUP(F8/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>66</v>
-      </c>
-      <c r="H8" s="41" t="n">
-        <f aca="false">IF(OR(B8="",D8=""),"",D8*(1-'Meu custo por hora'!$B$28)-F8)</f>
+      <c r="I8" s="43" t="n">
+        <f aca="false">IF(OR(B8="",D8=""),"",D8*(1-'Meu custo por hora'!$B$28)-H8)</f>
         <v>10.6761058802629</v>
       </c>
-      <c r="I8" s="42" t="str">
-        <f aca="false">IF(OR(B8="",D8=""),"",IF(D8&gt;=G8,"OK: preço cobre custos e margem",IF(H8&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>OK: preço cobre custos e margem</v>
-      </c>
       <c r="J8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="37" t="n">
+      <c r="B9" s="38" t="n">
         <v>90</v>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="39" t="n">
         <v>18</v>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="39" t="n">
         <v>90</v>
       </c>
-      <c r="E9" s="39" t="n">
+      <c r="E9" s="40" t="n">
+        <f aca="false">IF(B9="","",ROUNDUP(H9/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>84</v>
+      </c>
+      <c r="F9" s="41" t="str">
+        <f aca="false">IF(OR(B9="",D9=""),"",IF(D9&gt;=E9,"OK: cobre custos e margem",IF(I9&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>OK: cobre custos e margem</v>
+      </c>
+      <c r="G9" s="42" t="n">
         <f aca="false">IF(B9="","",B9/60*'Meu custo por hora'!$B$25)</f>
         <v>53.4286729436845</v>
       </c>
-      <c r="F9" s="39" t="n">
-        <f aca="false">IF(B9="","",E9+C9)</f>
+      <c r="H9" s="42" t="n">
+        <f aca="false">IF(B9="","",G9+C9)</f>
         <v>71.4286729436845</v>
       </c>
-      <c r="G9" s="40" t="n">
-        <f aca="false">IF(B9="","",ROUNDUP(F9/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>84</v>
-      </c>
-      <c r="H9" s="41" t="n">
-        <f aca="false">IF(OR(B9="",D9=""),"",D9*(1-'Meu custo por hora'!$B$28)-F9)</f>
+      <c r="I9" s="43" t="n">
+        <f aca="false">IF(OR(B9="",D9=""),"",D9*(1-'Meu custo por hora'!$B$28)-H9)</f>
         <v>14.9713270563155</v>
       </c>
-      <c r="I9" s="42" t="str">
-        <f aca="false">IF(OR(B9="",D9=""),"",IF(D9&gt;=G9,"OK: preço cobre custos e margem",IF(H9&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>OK: preço cobre custos e margem</v>
-      </c>
       <c r="J9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="37" t="n">
+      <c r="B10" s="38" t="n">
         <v>150</v>
       </c>
-      <c r="C10" s="38" t="n">
+      <c r="C10" s="39" t="n">
         <v>35</v>
       </c>
-      <c r="D10" s="38" t="n">
+      <c r="D10" s="39" t="n">
         <v>180</v>
       </c>
-      <c r="E10" s="39" t="n">
+      <c r="E10" s="40" t="n">
+        <f aca="false">IF(B10="","",ROUNDUP(H10/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>145</v>
+      </c>
+      <c r="F10" s="41" t="str">
+        <f aca="false">IF(OR(B10="",D10=""),"",IF(D10&gt;=E10,"OK: cobre custos e margem",IF(I10&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>OK: cobre custos e margem</v>
+      </c>
+      <c r="G10" s="42" t="n">
         <f aca="false">IF(B10="","",B10/60*'Meu custo por hora'!$B$25)</f>
         <v>89.0477882394742</v>
       </c>
-      <c r="F10" s="39" t="n">
-        <f aca="false">IF(B10="","",E10+C10)</f>
+      <c r="H10" s="42" t="n">
+        <f aca="false">IF(B10="","",G10+C10)</f>
         <v>124.047788239474</v>
       </c>
-      <c r="G10" s="40" t="n">
-        <f aca="false">IF(B10="","",ROUNDUP(F10/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>145</v>
-      </c>
-      <c r="H10" s="41" t="n">
-        <f aca="false">IF(OR(B10="",D10=""),"",D10*(1-'Meu custo por hora'!$B$28)-F10)</f>
+      <c r="I10" s="43" t="n">
+        <f aca="false">IF(OR(B10="",D10=""),"",D10*(1-'Meu custo por hora'!$B$28)-H10)</f>
         <v>48.7522117605258</v>
       </c>
-      <c r="I10" s="42" t="str">
-        <f aca="false">IF(OR(B10="",D10=""),"",IF(D10&gt;=G10,"OK: preço cobre custos e margem",IF(H10&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>OK: preço cobre custos e margem</v>
-      </c>
       <c r="J10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="B11" s="37" t="n">
+      <c r="B11" s="38" t="n">
         <v>120</v>
       </c>
-      <c r="C11" s="38" t="n">
+      <c r="C11" s="39" t="n">
         <v>22</v>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="39" t="n">
         <v>120</v>
       </c>
-      <c r="E11" s="39" t="n">
+      <c r="E11" s="40" t="n">
+        <f aca="false">IF(B11="","",ROUNDUP(H11/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>109</v>
+      </c>
+      <c r="F11" s="41" t="str">
+        <f aca="false">IF(OR(B11="",D11=""),"",IF(D11&gt;=E11,"OK: cobre custos e margem",IF(I11&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>OK: cobre custos e margem</v>
+      </c>
+      <c r="G11" s="42" t="n">
         <f aca="false">IF(B11="","",B11/60*'Meu custo por hora'!$B$25)</f>
         <v>71.2382305915793</v>
       </c>
-      <c r="F11" s="39" t="n">
-        <f aca="false">IF(B11="","",E11+C11)</f>
+      <c r="H11" s="42" t="n">
+        <f aca="false">IF(B11="","",G11+C11)</f>
         <v>93.2382305915793</v>
       </c>
-      <c r="G11" s="40" t="n">
-        <f aca="false">IF(B11="","",ROUNDUP(F11/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>109</v>
-      </c>
-      <c r="H11" s="41" t="n">
-        <f aca="false">IF(OR(B11="",D11=""),"",D11*(1-'Meu custo por hora'!$B$28)-F11)</f>
+      <c r="I11" s="43" t="n">
+        <f aca="false">IF(OR(B11="",D11=""),"",D11*(1-'Meu custo por hora'!$B$28)-H11)</f>
         <v>21.9617694084207</v>
       </c>
-      <c r="I11" s="42" t="str">
-        <f aca="false">IF(OR(B11="",D11=""),"",IF(D11&gt;=G11,"OK: preço cobre custos e margem",IF(H11&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>OK: preço cobre custos e margem</v>
-      </c>
       <c r="J11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="37" t="n">
+      <c r="B12" s="38" t="n">
         <v>30</v>
       </c>
-      <c r="C12" s="38" t="n">
+      <c r="C12" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="38" t="n">
+      <c r="D12" s="39" t="n">
         <v>25</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="40" t="n">
+        <f aca="false">IF(B12="","",ROUNDUP(H12/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v>25</v>
+      </c>
+      <c r="F12" s="41" t="str">
+        <f aca="false">IF(OR(B12="",D12=""),"",IF(D12&gt;=E12,"OK: cobre custos e margem",IF(I12&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v>OK: cobre custos e margem</v>
+      </c>
+      <c r="G12" s="42" t="n">
         <f aca="false">IF(B12="","",B12/60*'Meu custo por hora'!$B$25)</f>
         <v>17.8095576478948</v>
       </c>
-      <c r="F12" s="39" t="n">
-        <f aca="false">IF(B12="","",E12+C12)</f>
+      <c r="H12" s="42" t="n">
+        <f aca="false">IF(B12="","",G12+C12)</f>
         <v>20.8095576478948</v>
       </c>
-      <c r="G12" s="40" t="n">
-        <f aca="false">IF(B12="","",ROUNDUP(F12/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>25</v>
-      </c>
-      <c r="H12" s="41" t="n">
-        <f aca="false">IF(OR(B12="",D12=""),"",D12*(1-'Meu custo por hora'!$B$28)-F12)</f>
+      <c r="I12" s="43" t="n">
+        <f aca="false">IF(OR(B12="",D12=""),"",D12*(1-'Meu custo por hora'!$B$28)-H12)</f>
         <v>3.19044235210517</v>
       </c>
-      <c r="I12" s="42" t="str">
-        <f aca="false">IF(OR(B12="",D12=""),"",IF(D12&gt;=G12,"OK: preço cobre custos e margem",IF(H12&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
-        <v>OK: preço cobre custos e margem</v>
-      </c>
       <c r="J12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39" t="str">
+      <c r="A13" s="37"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="40" t="str">
+        <f aca="false">IF(B13="","",ROUNDUP(H13/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F13" s="41" t="str">
+        <f aca="false">IF(OR(B13="",D13=""),"",IF(D13&gt;=E13,"OK: cobre custos e margem",IF(I13&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G13" s="42" t="str">
         <f aca="false">IF(B13="","",B13/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F13" s="39" t="str">
-        <f aca="false">IF(B13="","",E13+C13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="40" t="str">
-        <f aca="false">IF(B13="","",ROUNDUP(F13/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H13" s="41" t="str">
-        <f aca="false">IF(OR(B13="",D13=""),"",D13*(1-'Meu custo por hora'!$B$28)-F13)</f>
-        <v/>
-      </c>
-      <c r="I13" s="42" t="str">
-        <f aca="false">IF(OR(B13="",D13=""),"",IF(D13&gt;=G13,"OK: preço cobre custos e margem",IF(H13&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H13" s="42" t="str">
+        <f aca="false">IF(B13="","",G13+C13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="43" t="str">
+        <f aca="false">IF(OR(B13="",D13=""),"",D13*(1-'Meu custo por hora'!$B$28)-H13)</f>
         <v/>
       </c>
       <c r="J13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39" t="str">
+      <c r="A14" s="37"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="40" t="str">
+        <f aca="false">IF(B14="","",ROUNDUP(H14/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F14" s="41" t="str">
+        <f aca="false">IF(OR(B14="",D14=""),"",IF(D14&gt;=E14,"OK: cobre custos e margem",IF(I14&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G14" s="42" t="str">
         <f aca="false">IF(B14="","",B14/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F14" s="39" t="str">
-        <f aca="false">IF(B14="","",E14+C14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="40" t="str">
-        <f aca="false">IF(B14="","",ROUNDUP(F14/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H14" s="41" t="str">
-        <f aca="false">IF(OR(B14="",D14=""),"",D14*(1-'Meu custo por hora'!$B$28)-F14)</f>
-        <v/>
-      </c>
-      <c r="I14" s="42" t="str">
-        <f aca="false">IF(OR(B14="",D14=""),"",IF(D14&gt;=G14,"OK: preço cobre custos e margem",IF(H14&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H14" s="42" t="str">
+        <f aca="false">IF(B14="","",G14+C14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="43" t="str">
+        <f aca="false">IF(OR(B14="",D14=""),"",D14*(1-'Meu custo por hora'!$B$28)-H14)</f>
         <v/>
       </c>
       <c r="J14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="39" t="str">
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="40" t="str">
+        <f aca="false">IF(B15="","",ROUNDUP(H15/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F15" s="41" t="str">
+        <f aca="false">IF(OR(B15="",D15=""),"",IF(D15&gt;=E15,"OK: cobre custos e margem",IF(I15&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G15" s="42" t="str">
         <f aca="false">IF(B15="","",B15/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F15" s="39" t="str">
-        <f aca="false">IF(B15="","",E15+C15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="40" t="str">
-        <f aca="false">IF(B15="","",ROUNDUP(F15/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H15" s="41" t="str">
-        <f aca="false">IF(OR(B15="",D15=""),"",D15*(1-'Meu custo por hora'!$B$28)-F15)</f>
-        <v/>
-      </c>
-      <c r="I15" s="42" t="str">
-        <f aca="false">IF(OR(B15="",D15=""),"",IF(D15&gt;=G15,"OK: preço cobre custos e margem",IF(H15&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H15" s="42" t="str">
+        <f aca="false">IF(B15="","",G15+C15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="43" t="str">
+        <f aca="false">IF(OR(B15="",D15=""),"",D15*(1-'Meu custo por hora'!$B$28)-H15)</f>
         <v/>
       </c>
       <c r="J15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="39" t="str">
+      <c r="A16" s="37"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="40" t="str">
+        <f aca="false">IF(B16="","",ROUNDUP(H16/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F16" s="41" t="str">
+        <f aca="false">IF(OR(B16="",D16=""),"",IF(D16&gt;=E16,"OK: cobre custos e margem",IF(I16&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G16" s="42" t="str">
         <f aca="false">IF(B16="","",B16/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F16" s="39" t="str">
-        <f aca="false">IF(B16="","",E16+C16)</f>
-        <v/>
-      </c>
-      <c r="G16" s="40" t="str">
-        <f aca="false">IF(B16="","",ROUNDUP(F16/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H16" s="41" t="str">
-        <f aca="false">IF(OR(B16="",D16=""),"",D16*(1-'Meu custo por hora'!$B$28)-F16)</f>
-        <v/>
-      </c>
-      <c r="I16" s="42" t="str">
-        <f aca="false">IF(OR(B16="",D16=""),"",IF(D16&gt;=G16,"OK: preço cobre custos e margem",IF(H16&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H16" s="42" t="str">
+        <f aca="false">IF(B16="","",G16+C16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="43" t="str">
+        <f aca="false">IF(OR(B16="",D16=""),"",D16*(1-'Meu custo por hora'!$B$28)-H16)</f>
         <v/>
       </c>
       <c r="J16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="39" t="str">
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="40" t="str">
+        <f aca="false">IF(B17="","",ROUNDUP(H17/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F17" s="41" t="str">
+        <f aca="false">IF(OR(B17="",D17=""),"",IF(D17&gt;=E17,"OK: cobre custos e margem",IF(I17&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G17" s="42" t="str">
         <f aca="false">IF(B17="","",B17/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F17" s="39" t="str">
-        <f aca="false">IF(B17="","",E17+C17)</f>
-        <v/>
-      </c>
-      <c r="G17" s="40" t="str">
-        <f aca="false">IF(B17="","",ROUNDUP(F17/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H17" s="41" t="str">
-        <f aca="false">IF(OR(B17="",D17=""),"",D17*(1-'Meu custo por hora'!$B$28)-F17)</f>
-        <v/>
-      </c>
-      <c r="I17" s="42" t="str">
-        <f aca="false">IF(OR(B17="",D17=""),"",IF(D17&gt;=G17,"OK: preço cobre custos e margem",IF(H17&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H17" s="42" t="str">
+        <f aca="false">IF(B17="","",G17+C17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="43" t="str">
+        <f aca="false">IF(OR(B17="",D17=""),"",D17*(1-'Meu custo por hora'!$B$28)-H17)</f>
         <v/>
       </c>
       <c r="J17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="39" t="str">
+      <c r="A18" s="37"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="40" t="str">
+        <f aca="false">IF(B18="","",ROUNDUP(H18/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F18" s="41" t="str">
+        <f aca="false">IF(OR(B18="",D18=""),"",IF(D18&gt;=E18,"OK: cobre custos e margem",IF(I18&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G18" s="42" t="str">
         <f aca="false">IF(B18="","",B18/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F18" s="39" t="str">
-        <f aca="false">IF(B18="","",E18+C18)</f>
-        <v/>
-      </c>
-      <c r="G18" s="40" t="str">
-        <f aca="false">IF(B18="","",ROUNDUP(F18/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H18" s="41" t="str">
-        <f aca="false">IF(OR(B18="",D18=""),"",D18*(1-'Meu custo por hora'!$B$28)-F18)</f>
-        <v/>
-      </c>
-      <c r="I18" s="42" t="str">
-        <f aca="false">IF(OR(B18="",D18=""),"",IF(D18&gt;=G18,"OK: preço cobre custos e margem",IF(H18&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H18" s="42" t="str">
+        <f aca="false">IF(B18="","",G18+C18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="43" t="str">
+        <f aca="false">IF(OR(B18="",D18=""),"",D18*(1-'Meu custo por hora'!$B$28)-H18)</f>
         <v/>
       </c>
       <c r="J18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39" t="str">
+      <c r="A19" s="37"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="40" t="str">
+        <f aca="false">IF(B19="","",ROUNDUP(H19/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F19" s="41" t="str">
+        <f aca="false">IF(OR(B19="",D19=""),"",IF(D19&gt;=E19,"OK: cobre custos e margem",IF(I19&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G19" s="42" t="str">
         <f aca="false">IF(B19="","",B19/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F19" s="39" t="str">
-        <f aca="false">IF(B19="","",E19+C19)</f>
-        <v/>
-      </c>
-      <c r="G19" s="40" t="str">
-        <f aca="false">IF(B19="","",ROUNDUP(F19/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H19" s="41" t="str">
-        <f aca="false">IF(OR(B19="",D19=""),"",D19*(1-'Meu custo por hora'!$B$28)-F19)</f>
-        <v/>
-      </c>
-      <c r="I19" s="42" t="str">
-        <f aca="false">IF(OR(B19="",D19=""),"",IF(D19&gt;=G19,"OK: preço cobre custos e margem",IF(H19&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H19" s="42" t="str">
+        <f aca="false">IF(B19="","",G19+C19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="43" t="str">
+        <f aca="false">IF(OR(B19="",D19=""),"",D19*(1-'Meu custo por hora'!$B$28)-H19)</f>
         <v/>
       </c>
       <c r="J19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="39" t="str">
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="40" t="str">
+        <f aca="false">IF(B20="","",ROUNDUP(H20/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F20" s="41" t="str">
+        <f aca="false">IF(OR(B20="",D20=""),"",IF(D20&gt;=E20,"OK: cobre custos e margem",IF(I20&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G20" s="42" t="str">
         <f aca="false">IF(B20="","",B20/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F20" s="39" t="str">
-        <f aca="false">IF(B20="","",E20+C20)</f>
-        <v/>
-      </c>
-      <c r="G20" s="40" t="str">
-        <f aca="false">IF(B20="","",ROUNDUP(F20/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H20" s="41" t="str">
-        <f aca="false">IF(OR(B20="",D20=""),"",D20*(1-'Meu custo por hora'!$B$28)-F20)</f>
-        <v/>
-      </c>
-      <c r="I20" s="42" t="str">
-        <f aca="false">IF(OR(B20="",D20=""),"",IF(D20&gt;=G20,"OK: preço cobre custos e margem",IF(H20&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H20" s="42" t="str">
+        <f aca="false">IF(B20="","",G20+C20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="43" t="str">
+        <f aca="false">IF(OR(B20="",D20=""),"",D20*(1-'Meu custo por hora'!$B$28)-H20)</f>
         <v/>
       </c>
       <c r="J20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="39" t="str">
+      <c r="A21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="40" t="str">
+        <f aca="false">IF(B21="","",ROUNDUP(H21/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F21" s="41" t="str">
+        <f aca="false">IF(OR(B21="",D21=""),"",IF(D21&gt;=E21,"OK: cobre custos e margem",IF(I21&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G21" s="42" t="str">
         <f aca="false">IF(B21="","",B21/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F21" s="39" t="str">
-        <f aca="false">IF(B21="","",E21+C21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="40" t="str">
-        <f aca="false">IF(B21="","",ROUNDUP(F21/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H21" s="41" t="str">
-        <f aca="false">IF(OR(B21="",D21=""),"",D21*(1-'Meu custo por hora'!$B$28)-F21)</f>
-        <v/>
-      </c>
-      <c r="I21" s="42" t="str">
-        <f aca="false">IF(OR(B21="",D21=""),"",IF(D21&gt;=G21,"OK: preço cobre custos e margem",IF(H21&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H21" s="42" t="str">
+        <f aca="false">IF(B21="","",G21+C21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="43" t="str">
+        <f aca="false">IF(OR(B21="",D21=""),"",D21*(1-'Meu custo por hora'!$B$28)-H21)</f>
         <v/>
       </c>
       <c r="J21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="36"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39" t="str">
+      <c r="A22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="40" t="str">
+        <f aca="false">IF(B22="","",ROUNDUP(H22/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F22" s="41" t="str">
+        <f aca="false">IF(OR(B22="",D22=""),"",IF(D22&gt;=E22,"OK: cobre custos e margem",IF(I22&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G22" s="42" t="str">
         <f aca="false">IF(B22="","",B22/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F22" s="39" t="str">
-        <f aca="false">IF(B22="","",E22+C22)</f>
-        <v/>
-      </c>
-      <c r="G22" s="40" t="str">
-        <f aca="false">IF(B22="","",ROUNDUP(F22/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H22" s="41" t="str">
-        <f aca="false">IF(OR(B22="",D22=""),"",D22*(1-'Meu custo por hora'!$B$28)-F22)</f>
-        <v/>
-      </c>
-      <c r="I22" s="42" t="str">
-        <f aca="false">IF(OR(B22="",D22=""),"",IF(D22&gt;=G22,"OK: preço cobre custos e margem",IF(H22&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H22" s="42" t="str">
+        <f aca="false">IF(B22="","",G22+C22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="43" t="str">
+        <f aca="false">IF(OR(B22="",D22=""),"",D22*(1-'Meu custo por hora'!$B$28)-H22)</f>
         <v/>
       </c>
       <c r="J22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="39" t="str">
+      <c r="A23" s="37"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="40" t="str">
+        <f aca="false">IF(B23="","",ROUNDUP(H23/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F23" s="41" t="str">
+        <f aca="false">IF(OR(B23="",D23=""),"",IF(D23&gt;=E23,"OK: cobre custos e margem",IF(I23&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G23" s="42" t="str">
         <f aca="false">IF(B23="","",B23/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F23" s="39" t="str">
-        <f aca="false">IF(B23="","",E23+C23)</f>
-        <v/>
-      </c>
-      <c r="G23" s="40" t="str">
-        <f aca="false">IF(B23="","",ROUNDUP(F23/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H23" s="41" t="str">
-        <f aca="false">IF(OR(B23="",D23=""),"",D23*(1-'Meu custo por hora'!$B$28)-F23)</f>
-        <v/>
-      </c>
-      <c r="I23" s="42" t="str">
-        <f aca="false">IF(OR(B23="",D23=""),"",IF(D23&gt;=G23,"OK: preço cobre custos e margem",IF(H23&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H23" s="42" t="str">
+        <f aca="false">IF(B23="","",G23+C23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="43" t="str">
+        <f aca="false">IF(OR(B23="",D23=""),"",D23*(1-'Meu custo por hora'!$B$28)-H23)</f>
         <v/>
       </c>
       <c r="J23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="39" t="str">
+      <c r="A24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="40" t="str">
+        <f aca="false">IF(B24="","",ROUNDUP(H24/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F24" s="41" t="str">
+        <f aca="false">IF(OR(B24="",D24=""),"",IF(D24&gt;=E24,"OK: cobre custos e margem",IF(I24&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G24" s="42" t="str">
         <f aca="false">IF(B24="","",B24/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F24" s="39" t="str">
-        <f aca="false">IF(B24="","",E24+C24)</f>
-        <v/>
-      </c>
-      <c r="G24" s="40" t="str">
-        <f aca="false">IF(B24="","",ROUNDUP(F24/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H24" s="41" t="str">
-        <f aca="false">IF(OR(B24="",D24=""),"",D24*(1-'Meu custo por hora'!$B$28)-F24)</f>
-        <v/>
-      </c>
-      <c r="I24" s="42" t="str">
-        <f aca="false">IF(OR(B24="",D24=""),"",IF(D24&gt;=G24,"OK: preço cobre custos e margem",IF(H24&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H24" s="42" t="str">
+        <f aca="false">IF(B24="","",G24+C24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="43" t="str">
+        <f aca="false">IF(OR(B24="",D24=""),"",D24*(1-'Meu custo por hora'!$B$28)-H24)</f>
         <v/>
       </c>
       <c r="J24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39" t="str">
+      <c r="A25" s="37"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="40" t="str">
+        <f aca="false">IF(B25="","",ROUNDUP(H25/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F25" s="41" t="str">
+        <f aca="false">IF(OR(B25="",D25=""),"",IF(D25&gt;=E25,"OK: cobre custos e margem",IF(I25&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G25" s="42" t="str">
         <f aca="false">IF(B25="","",B25/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F25" s="39" t="str">
-        <f aca="false">IF(B25="","",E25+C25)</f>
-        <v/>
-      </c>
-      <c r="G25" s="40" t="str">
-        <f aca="false">IF(B25="","",ROUNDUP(F25/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H25" s="41" t="str">
-        <f aca="false">IF(OR(B25="",D25=""),"",D25*(1-'Meu custo por hora'!$B$28)-F25)</f>
-        <v/>
-      </c>
-      <c r="I25" s="42" t="str">
-        <f aca="false">IF(OR(B25="",D25=""),"",IF(D25&gt;=G25,"OK: preço cobre custos e margem",IF(H25&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H25" s="42" t="str">
+        <f aca="false">IF(B25="","",G25+C25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="43" t="str">
+        <f aca="false">IF(OR(B25="",D25=""),"",D25*(1-'Meu custo por hora'!$B$28)-H25)</f>
         <v/>
       </c>
       <c r="J25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="36"/>
-      <c r="B26" s="37"/>
-      <c r="C26" s="38"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="39" t="str">
+      <c r="A26" s="37"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="40" t="str">
+        <f aca="false">IF(B26="","",ROUNDUP(H26/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F26" s="41" t="str">
+        <f aca="false">IF(OR(B26="",D26=""),"",IF(D26&gt;=E26,"OK: cobre custos e margem",IF(I26&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G26" s="42" t="str">
         <f aca="false">IF(B26="","",B26/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F26" s="39" t="str">
-        <f aca="false">IF(B26="","",E26+C26)</f>
-        <v/>
-      </c>
-      <c r="G26" s="40" t="str">
-        <f aca="false">IF(B26="","",ROUNDUP(F26/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H26" s="41" t="str">
-        <f aca="false">IF(OR(B26="",D26=""),"",D26*(1-'Meu custo por hora'!$B$28)-F26)</f>
-        <v/>
-      </c>
-      <c r="I26" s="42" t="str">
-        <f aca="false">IF(OR(B26="",D26=""),"",IF(D26&gt;=G26,"OK: preço cobre custos e margem",IF(H26&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H26" s="42" t="str">
+        <f aca="false">IF(B26="","",G26+C26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="43" t="str">
+        <f aca="false">IF(OR(B26="",D26=""),"",D26*(1-'Meu custo por hora'!$B$28)-H26)</f>
         <v/>
       </c>
       <c r="J26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="36"/>
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="39" t="str">
+      <c r="A27" s="37"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="40" t="str">
+        <f aca="false">IF(B27="","",ROUNDUP(H27/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F27" s="41" t="str">
+        <f aca="false">IF(OR(B27="",D27=""),"",IF(D27&gt;=E27,"OK: cobre custos e margem",IF(I27&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G27" s="42" t="str">
         <f aca="false">IF(B27="","",B27/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F27" s="39" t="str">
-        <f aca="false">IF(B27="","",E27+C27)</f>
-        <v/>
-      </c>
-      <c r="G27" s="40" t="str">
-        <f aca="false">IF(B27="","",ROUNDUP(F27/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H27" s="41" t="str">
-        <f aca="false">IF(OR(B27="",D27=""),"",D27*(1-'Meu custo por hora'!$B$28)-F27)</f>
-        <v/>
-      </c>
-      <c r="I27" s="42" t="str">
-        <f aca="false">IF(OR(B27="",D27=""),"",IF(D27&gt;=G27,"OK: preço cobre custos e margem",IF(H27&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H27" s="42" t="str">
+        <f aca="false">IF(B27="","",G27+C27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="43" t="str">
+        <f aca="false">IF(OR(B27="",D27=""),"",D27*(1-'Meu custo por hora'!$B$28)-H27)</f>
         <v/>
       </c>
       <c r="J27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="36"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="39" t="str">
+      <c r="A28" s="37"/>
+      <c r="B28" s="38"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="40" t="str">
+        <f aca="false">IF(B28="","",ROUNDUP(H28/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F28" s="41" t="str">
+        <f aca="false">IF(OR(B28="",D28=""),"",IF(D28&gt;=E28,"OK: cobre custos e margem",IF(I28&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G28" s="42" t="str">
         <f aca="false">IF(B28="","",B28/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F28" s="39" t="str">
-        <f aca="false">IF(B28="","",E28+C28)</f>
-        <v/>
-      </c>
-      <c r="G28" s="40" t="str">
-        <f aca="false">IF(B28="","",ROUNDUP(F28/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H28" s="41" t="str">
-        <f aca="false">IF(OR(B28="",D28=""),"",D28*(1-'Meu custo por hora'!$B$28)-F28)</f>
-        <v/>
-      </c>
-      <c r="I28" s="42" t="str">
-        <f aca="false">IF(OR(B28="",D28=""),"",IF(D28&gt;=G28,"OK: preço cobre custos e margem",IF(H28&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H28" s="42" t="str">
+        <f aca="false">IF(B28="","",G28+C28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="43" t="str">
+        <f aca="false">IF(OR(B28="",D28=""),"",D28*(1-'Meu custo por hora'!$B$28)-H28)</f>
         <v/>
       </c>
       <c r="J28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="36"/>
-      <c r="B29" s="37"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="39" t="str">
+      <c r="A29" s="37"/>
+      <c r="B29" s="38"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="40" t="str">
+        <f aca="false">IF(B29="","",ROUNDUP(H29/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
+        <v/>
+      </c>
+      <c r="F29" s="41" t="str">
+        <f aca="false">IF(OR(B29="",D29=""),"",IF(D29&gt;=E29,"OK: cobre custos e margem",IF(I29&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
+        <v/>
+      </c>
+      <c r="G29" s="42" t="str">
         <f aca="false">IF(B29="","",B29/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="F29" s="39" t="str">
-        <f aca="false">IF(B29="","",E29+C29)</f>
-        <v/>
-      </c>
-      <c r="G29" s="40" t="str">
-        <f aca="false">IF(B29="","",ROUNDUP(F29/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v/>
-      </c>
-      <c r="H29" s="41" t="str">
-        <f aca="false">IF(OR(B29="",D29=""),"",D29*(1-'Meu custo por hora'!$B$28)-F29)</f>
-        <v/>
-      </c>
-      <c r="I29" s="42" t="str">
-        <f aca="false">IF(OR(B29="",D29=""),"",IF(D29&gt;=G29,"OK: preço cobre custos e margem",IF(H29&gt;=0,"Atenção: pouca folga","PREJUÍZO: preço abaixo do custo")))</f>
+      <c r="H29" s="42" t="str">
+        <f aca="false">IF(B29="","",G29+C29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="43" t="str">
+        <f aca="false">IF(OR(B29="",D29=""),"",D29*(1-'Meu custo por hora'!$B$28)-H29)</f>
         <v/>
       </c>
       <c r="J29" s="6"/>
@@ -3659,59 +3661,59 @@
       <c r="J30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="43" t="s">
+      <c r="A31" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="43"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="43"/>
-      <c r="I31" s="43"/>
+      <c r="B31" s="44"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
       <c r="J31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="43"/>
-      <c r="I32" s="43"/>
+      <c r="B32" s="44"/>
+      <c r="C32" s="44"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
       <c r="J32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="43" t="s">
+      <c r="A33" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="B33" s="43"/>
-      <c r="C33" s="43"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="43"/>
-      <c r="I33" s="43"/>
+      <c r="B33" s="44"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="44"/>
       <c r="J33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="43"/>
+      <c r="B34" s="44"/>
+      <c r="C34" s="44"/>
+      <c r="D34" s="44"/>
+      <c r="E34" s="44"/>
+      <c r="F34" s="44"/>
+      <c r="G34" s="44"/>
+      <c r="H34" s="44"/>
+      <c r="I34" s="44"/>
       <c r="J34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3760,15 +3762,15 @@
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A34:I34"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I29">
+  <conditionalFormatting sqref="F5:F29">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>LEFT($I5,2)="OK"</formula>
+      <formula>LEFT($F5,2)="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>LEFT($I5,7)="Atenção"</formula>
+      <formula>LEFT($F5,7)="Atenção"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>LEFT($I5,4)="PREJ"</formula>
+      <formula>LEFT($F5,4)="PREJ"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -3875,78 +3877,78 @@
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6"/>
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44" t="s">
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44" t="s">
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-      <c r="K5" s="44" t="s">
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="45" t="s">
         <v>89</v>
       </c>
-      <c r="L5" s="44"/>
-      <c r="M5" s="44"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
       <c r="N5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="46" t="n">
         <f aca="false">'Meu custo por hora'!B25</f>
         <v>35.6191152957897</v>
       </c>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="46" t="n">
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="47" t="n">
         <f aca="false">COUNT('Meus serviços'!B5:B29)</f>
         <v>8</v>
       </c>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46" t="n">
-        <f aca="false">COUNTIF('Meus serviços'!I5:I29,"Atenção*")+COUNTIF('Meus serviços'!I5:I29,"PREJUÍZO*")</f>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47" t="n">
+        <f aca="false">COUNTIF('Meus serviços'!F5:F29,"Atenção*")+COUNTIF('Meus serviços'!F5:F29,"PREJUÍZO*")</f>
         <v>3</v>
       </c>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="47" t="n">
-        <f aca="false">COUNTIF('Meus serviços'!I5:I29,"PREJUÍZO*")</f>
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="48" t="n">
+        <f aca="false">COUNTIF('Meus serviços'!F5:F29,"PREJUÍZO*")</f>
         <v>2</v>
       </c>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="48"/>
       <c r="N6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48" t="s">
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48" t="s">
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="48"/>
-      <c r="K7" s="48" t="s">
+      <c r="I7" s="49"/>
+      <c r="J7" s="49"/>
+      <c r="K7" s="49" t="s">
         <v>93</v>
       </c>
-      <c r="L7" s="48"/>
-      <c r="M7" s="48"/>
+      <c r="L7" s="49"/>
+      <c r="M7" s="49"/>
       <c r="N7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3967,21 +3969,21 @@
     </row>
     <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
-      <c r="B9" s="49" t="str">
+      <c r="B9" s="50" t="str">
         <f aca="false">IF(K6&gt;0,"Atenção: "&amp;K6&amp;" serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.",IF(H6&gt;0,"Alguns serviços têm pouca folga. Compare o preço de hoje com o preço sugerido.","Os preços cadastrados cobrem seus custos e a margem. Revise quando seus gastos mudarem."))</f>
         <v>Atenção: 2 serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.</v>
       </c>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="49"/>
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
       <c r="N9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4340,20 +4342,20 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6"/>
-      <c r="B32" s="43" t="s">
+      <c r="B32" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="43"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="43"/>
-      <c r="I32" s="43"/>
-      <c r="J32" s="43"/>
-      <c r="K32" s="43"/>
-      <c r="L32" s="43"/>
-      <c r="M32" s="43"/>
+      <c r="C32" s="44"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44"/>
+      <c r="K32" s="44"/>
+      <c r="L32" s="44"/>
+      <c r="M32" s="44"/>
       <c r="N32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4483,10 +4485,10 @@
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6"/>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="51" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="50"/>
+      <c r="C3" s="51"/>
       <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4497,310 +4499,310 @@
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6"/>
-      <c r="B5" s="51" t="s">
+      <c r="B5" s="52" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="53" t="s">
         <v>98</v>
       </c>
       <c r="D5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
-      <c r="B6" s="53" t="str">
+      <c r="B6" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B5="","",'Meus serviços'!A5)</f>
         <v>Esmaltação simples (mão)</v>
       </c>
-      <c r="C6" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B5="","",IF('Meus serviços'!D5&gt;='Meus serviços'!G5,'Meus serviços'!D5,'Meus serviços'!G5))</f>
+      <c r="C6" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B5="","",IF('Meus serviços'!D5&gt;='Meus serviços'!E5,'Meus serviços'!D5,'Meus serviços'!E5))</f>
         <v>36</v>
       </c>
       <c r="D6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
-      <c r="B7" s="53" t="str">
+      <c r="B7" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B6="","",'Meus serviços'!A6)</f>
         <v>Esmaltação simples (pé)</v>
       </c>
-      <c r="C7" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B6="","",IF('Meus serviços'!D6&gt;='Meus serviços'!G6,'Meus serviços'!D6,'Meus serviços'!G6))</f>
+      <c r="C7" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B6="","",IF('Meus serviços'!D6&gt;='Meus serviços'!E6,'Meus serviços'!D6,'Meus serviços'!E6))</f>
         <v>40</v>
       </c>
       <c r="D7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6"/>
-      <c r="B8" s="53" t="str">
+      <c r="B8" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B7="","",'Meus serviços'!A7)</f>
         <v>Mão + pé</v>
       </c>
-      <c r="C8" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B7="","",IF('Meus serviços'!D7&gt;='Meus serviços'!G7,'Meus serviços'!D7,'Meus serviços'!G7))</f>
+      <c r="C8" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B7="","",IF('Meus serviços'!D7&gt;='Meus serviços'!E7,'Meus serviços'!D7,'Meus serviços'!E7))</f>
         <v>72</v>
       </c>
       <c r="D8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
-      <c r="B9" s="53" t="str">
+      <c r="B9" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B8="","",'Meus serviços'!A8)</f>
         <v>Esmaltação em gel (mão)</v>
       </c>
-      <c r="C9" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B8="","",IF('Meus serviços'!D8&gt;='Meus serviços'!G8,'Meus serviços'!D8,'Meus serviços'!G8))</f>
+      <c r="C9" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B8="","",IF('Meus serviços'!D8&gt;='Meus serviços'!E8,'Meus serviços'!D8,'Meus serviços'!E8))</f>
         <v>70</v>
       </c>
       <c r="D9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6"/>
-      <c r="B10" s="53" t="str">
+      <c r="B10" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B9="","",'Meus serviços'!A9)</f>
         <v>Blindagem</v>
       </c>
-      <c r="C10" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B9="","",IF('Meus serviços'!D9&gt;='Meus serviços'!G9,'Meus serviços'!D9,'Meus serviços'!G9))</f>
+      <c r="C10" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B9="","",IF('Meus serviços'!D9&gt;='Meus serviços'!E9,'Meus serviços'!D9,'Meus serviços'!E9))</f>
         <v>90</v>
       </c>
       <c r="D10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
-      <c r="B11" s="53" t="str">
+      <c r="B11" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B10="","",'Meus serviços'!A10)</f>
         <v>Alongamento em gel</v>
       </c>
-      <c r="C11" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B10="","",IF('Meus serviços'!D10&gt;='Meus serviços'!G10,'Meus serviços'!D10,'Meus serviços'!G10))</f>
+      <c r="C11" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B10="","",IF('Meus serviços'!D10&gt;='Meus serviços'!E10,'Meus serviços'!D10,'Meus serviços'!E10))</f>
         <v>180</v>
       </c>
       <c r="D11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
-      <c r="B12" s="53" t="str">
+      <c r="B12" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B11="","",'Meus serviços'!A11)</f>
         <v>Manutenção de alongamento</v>
       </c>
-      <c r="C12" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B11="","",IF('Meus serviços'!D11&gt;='Meus serviços'!G11,'Meus serviços'!D11,'Meus serviços'!G11))</f>
+      <c r="C12" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B11="","",IF('Meus serviços'!D11&gt;='Meus serviços'!E11,'Meus serviços'!D11,'Meus serviços'!E11))</f>
         <v>120</v>
       </c>
       <c r="D12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6"/>
-      <c r="B13" s="53" t="str">
+      <c r="B13" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B12="","",'Meus serviços'!A12)</f>
         <v>Remoção</v>
       </c>
-      <c r="C13" s="54" t="n">
-        <f aca="false">IF('Meus serviços'!B12="","",IF('Meus serviços'!D12&gt;='Meus serviços'!G12,'Meus serviços'!D12,'Meus serviços'!G12))</f>
+      <c r="C13" s="55" t="n">
+        <f aca="false">IF('Meus serviços'!B12="","",IF('Meus serviços'!D12&gt;='Meus serviços'!E12,'Meus serviços'!D12,'Meus serviços'!E12))</f>
         <v>25</v>
       </c>
       <c r="D13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
-      <c r="B14" s="53" t="str">
+      <c r="B14" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B13="","",'Meus serviços'!A13)</f>
         <v/>
       </c>
-      <c r="C14" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B13="","",IF('Meus serviços'!D13&gt;='Meus serviços'!G13,'Meus serviços'!D13,'Meus serviços'!G13))</f>
+      <c r="C14" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B13="","",IF('Meus serviços'!D13&gt;='Meus serviços'!E13,'Meus serviços'!D13,'Meus serviços'!E13))</f>
         <v/>
       </c>
       <c r="D14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
-      <c r="B15" s="53" t="str">
+      <c r="B15" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B14="","",'Meus serviços'!A14)</f>
         <v/>
       </c>
-      <c r="C15" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B14="","",IF('Meus serviços'!D14&gt;='Meus serviços'!G14,'Meus serviços'!D14,'Meus serviços'!G14))</f>
+      <c r="C15" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B14="","",IF('Meus serviços'!D14&gt;='Meus serviços'!E14,'Meus serviços'!D14,'Meus serviços'!E14))</f>
         <v/>
       </c>
       <c r="D15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6"/>
-      <c r="B16" s="53" t="str">
+      <c r="B16" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B15="","",'Meus serviços'!A15)</f>
         <v/>
       </c>
-      <c r="C16" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B15="","",IF('Meus serviços'!D15&gt;='Meus serviços'!G15,'Meus serviços'!D15,'Meus serviços'!G15))</f>
+      <c r="C16" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B15="","",IF('Meus serviços'!D15&gt;='Meus serviços'!E15,'Meus serviços'!D15,'Meus serviços'!E15))</f>
         <v/>
       </c>
       <c r="D16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
-      <c r="B17" s="53" t="str">
+      <c r="B17" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B16="","",'Meus serviços'!A16)</f>
         <v/>
       </c>
-      <c r="C17" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B16="","",IF('Meus serviços'!D16&gt;='Meus serviços'!G16,'Meus serviços'!D16,'Meus serviços'!G16))</f>
+      <c r="C17" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B16="","",IF('Meus serviços'!D16&gt;='Meus serviços'!E16,'Meus serviços'!D16,'Meus serviços'!E16))</f>
         <v/>
       </c>
       <c r="D17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
-      <c r="B18" s="53" t="str">
+      <c r="B18" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B17="","",'Meus serviços'!A17)</f>
         <v/>
       </c>
-      <c r="C18" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B17="","",IF('Meus serviços'!D17&gt;='Meus serviços'!G17,'Meus serviços'!D17,'Meus serviços'!G17))</f>
+      <c r="C18" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B17="","",IF('Meus serviços'!D17&gt;='Meus serviços'!E17,'Meus serviços'!D17,'Meus serviços'!E17))</f>
         <v/>
       </c>
       <c r="D18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6"/>
-      <c r="B19" s="53" t="str">
+      <c r="B19" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B18="","",'Meus serviços'!A18)</f>
         <v/>
       </c>
-      <c r="C19" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B18="","",IF('Meus serviços'!D18&gt;='Meus serviços'!G18,'Meus serviços'!D18,'Meus serviços'!G18))</f>
+      <c r="C19" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B18="","",IF('Meus serviços'!D18&gt;='Meus serviços'!E18,'Meus serviços'!D18,'Meus serviços'!E18))</f>
         <v/>
       </c>
       <c r="D19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
-      <c r="B20" s="53" t="str">
+      <c r="B20" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B19="","",'Meus serviços'!A19)</f>
         <v/>
       </c>
-      <c r="C20" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B19="","",IF('Meus serviços'!D19&gt;='Meus serviços'!G19,'Meus serviços'!D19,'Meus serviços'!G19))</f>
+      <c r="C20" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B19="","",IF('Meus serviços'!D19&gt;='Meus serviços'!E19,'Meus serviços'!D19,'Meus serviços'!E19))</f>
         <v/>
       </c>
       <c r="D20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6"/>
-      <c r="B21" s="53" t="str">
+      <c r="B21" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B20="","",'Meus serviços'!A20)</f>
         <v/>
       </c>
-      <c r="C21" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B20="","",IF('Meus serviços'!D20&gt;='Meus serviços'!G20,'Meus serviços'!D20,'Meus serviços'!G20))</f>
+      <c r="C21" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B20="","",IF('Meus serviços'!D20&gt;='Meus serviços'!E20,'Meus serviços'!D20,'Meus serviços'!E20))</f>
         <v/>
       </c>
       <c r="D21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6"/>
-      <c r="B22" s="53" t="str">
+      <c r="B22" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B21="","",'Meus serviços'!A21)</f>
         <v/>
       </c>
-      <c r="C22" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B21="","",IF('Meus serviços'!D21&gt;='Meus serviços'!G21,'Meus serviços'!D21,'Meus serviços'!G21))</f>
+      <c r="C22" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B21="","",IF('Meus serviços'!D21&gt;='Meus serviços'!E21,'Meus serviços'!D21,'Meus serviços'!E21))</f>
         <v/>
       </c>
       <c r="D22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6"/>
-      <c r="B23" s="53" t="str">
+      <c r="B23" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B22="","",'Meus serviços'!A22)</f>
         <v/>
       </c>
-      <c r="C23" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B22="","",IF('Meus serviços'!D22&gt;='Meus serviços'!G22,'Meus serviços'!D22,'Meus serviços'!G22))</f>
+      <c r="C23" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B22="","",IF('Meus serviços'!D22&gt;='Meus serviços'!E22,'Meus serviços'!D22,'Meus serviços'!E22))</f>
         <v/>
       </c>
       <c r="D23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6"/>
-      <c r="B24" s="53" t="str">
+      <c r="B24" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B23="","",'Meus serviços'!A23)</f>
         <v/>
       </c>
-      <c r="C24" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B23="","",IF('Meus serviços'!D23&gt;='Meus serviços'!G23,'Meus serviços'!D23,'Meus serviços'!G23))</f>
+      <c r="C24" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B23="","",IF('Meus serviços'!D23&gt;='Meus serviços'!E23,'Meus serviços'!D23,'Meus serviços'!E23))</f>
         <v/>
       </c>
       <c r="D24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6"/>
-      <c r="B25" s="53" t="str">
+      <c r="B25" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B24="","",'Meus serviços'!A24)</f>
         <v/>
       </c>
-      <c r="C25" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B24="","",IF('Meus serviços'!D24&gt;='Meus serviços'!G24,'Meus serviços'!D24,'Meus serviços'!G24))</f>
+      <c r="C25" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B24="","",IF('Meus serviços'!D24&gt;='Meus serviços'!E24,'Meus serviços'!D24,'Meus serviços'!E24))</f>
         <v/>
       </c>
       <c r="D25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6"/>
-      <c r="B26" s="53" t="str">
+      <c r="B26" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B25="","",'Meus serviços'!A25)</f>
         <v/>
       </c>
-      <c r="C26" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B25="","",IF('Meus serviços'!D25&gt;='Meus serviços'!G25,'Meus serviços'!D25,'Meus serviços'!G25))</f>
+      <c r="C26" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B25="","",IF('Meus serviços'!D25&gt;='Meus serviços'!E25,'Meus serviços'!D25,'Meus serviços'!E25))</f>
         <v/>
       </c>
       <c r="D26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6"/>
-      <c r="B27" s="53" t="str">
+      <c r="B27" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B26="","",'Meus serviços'!A26)</f>
         <v/>
       </c>
-      <c r="C27" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B26="","",IF('Meus serviços'!D26&gt;='Meus serviços'!G26,'Meus serviços'!D26,'Meus serviços'!G26))</f>
+      <c r="C27" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B26="","",IF('Meus serviços'!D26&gt;='Meus serviços'!E26,'Meus serviços'!D26,'Meus serviços'!E26))</f>
         <v/>
       </c>
       <c r="D27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6"/>
-      <c r="B28" s="53" t="str">
+      <c r="B28" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B27="","",'Meus serviços'!A27)</f>
         <v/>
       </c>
-      <c r="C28" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B27="","",IF('Meus serviços'!D27&gt;='Meus serviços'!G27,'Meus serviços'!D27,'Meus serviços'!G27))</f>
+      <c r="C28" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B27="","",IF('Meus serviços'!D27&gt;='Meus serviços'!E27,'Meus serviços'!D27,'Meus serviços'!E27))</f>
         <v/>
       </c>
       <c r="D28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6"/>
-      <c r="B29" s="53" t="str">
+      <c r="B29" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B28="","",'Meus serviços'!A28)</f>
         <v/>
       </c>
-      <c r="C29" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B28="","",IF('Meus serviços'!D28&gt;='Meus serviços'!G28,'Meus serviços'!D28,'Meus serviços'!G28))</f>
+      <c r="C29" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B28="","",IF('Meus serviços'!D28&gt;='Meus serviços'!E28,'Meus serviços'!D28,'Meus serviços'!E28))</f>
         <v/>
       </c>
       <c r="D29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6"/>
-      <c r="B30" s="53" t="str">
+      <c r="B30" s="54" t="str">
         <f aca="false">IF('Meus serviços'!B29="","",'Meus serviços'!A29)</f>
         <v/>
       </c>
-      <c r="C30" s="54" t="str">
-        <f aca="false">IF('Meus serviços'!B29="","",IF('Meus serviços'!D29&gt;='Meus serviços'!G29,'Meus serviços'!D29,'Meus serviços'!G29))</f>
+      <c r="C30" s="55" t="str">
+        <f aca="false">IF('Meus serviços'!B29="","",IF('Meus serviços'!D29&gt;='Meus serviços'!E29,'Meus serviços'!D29,'Meus serviços'!E29))</f>
         <v/>
       </c>
       <c r="D30" s="6"/>
@@ -4821,10 +4823,10 @@
     </row>
     <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6"/>
-      <c r="B33" s="55" t="s">
+      <c r="B33" s="56" t="s">
         <v>99</v>
       </c>
-      <c r="C33" s="55"/>
+      <c r="C33" s="56"/>
       <c r="D33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Calculadora web mobile (calculadora.html), links na pagina de obrigado e FAQ, coluna B da planilha mais larga
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -1477,11 +1477,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="16946007"/>
-        <c:axId val="14740886"/>
+        <c:axId val="50455225"/>
+        <c:axId val="11777598"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="16946007"/>
+        <c:axId val="50455225"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1513,7 +1513,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14740886"/>
+        <c:crossAx val="11777598"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1521,7 +1521,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14740886"/>
+        <c:axId val="11777598"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1563,7 +1563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16946007"/>
+        <c:crossAx val="50455225"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2475,7 +2475,7 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
   </cols>

</xml_diff>

<commit_message>
Planilha Excel e previas no visual novo (vinho, rosa e dourado)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -367,14 +367,14 @@
       <b val="true"/>
       <sz val="28"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="13"/>
-      <color rgb="FFF3E3B6"/>
+      <color rgb="FFFBE7A6"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -391,7 +391,7 @@
       <b val="true"/>
       <sz val="18"/>
       <color rgb="FF3A0A26"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -399,7 +399,7 @@
       <b val="true"/>
       <sz val="22"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -430,7 +430,7 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FF3A0A26"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -459,7 +459,7 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FFC9A24B"/>
+      <color rgb="FFE0B84C"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -468,7 +468,7 @@
       <b val="true"/>
       <sz val="20"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -522,7 +522,7 @@
       <b val="true"/>
       <sz val="18"/>
       <color rgb="FFC2185B"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -554,7 +554,7 @@
       <b val="true"/>
       <sz val="26"/>
       <color rgb="FFC2185B"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -562,7 +562,7 @@
       <b val="true"/>
       <sz val="26"/>
       <color rgb="FFB00040"/>
-      <name val="Georgia"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -598,7 +598,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -607,14 +607,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC2185B"/>
-        <bgColor rgb="FFB00040"/>
+        <fgColor rgb="FF5A1236"/>
+        <bgColor rgb="FF3A0A26"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC9A24B"/>
-        <bgColor rgb="FFFF9900"/>
+        <fgColor rgb="FFFF4FA3"/>
+        <bgColor rgb="FFE91E78"/>
       </patternFill>
     </fill>
     <fill>
@@ -631,8 +631,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3E3B6"/>
-        <bgColor rgb="FFFFF1CC"/>
+        <fgColor rgb="FFFBE7A6"/>
+        <bgColor rgb="FFFFF3C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -659,6 +659,12 @@
         <bgColor rgb="FFFCE9F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0B84C"/>
+        <bgColor rgb="FFFF9900"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="14">
     <border diagonalUp="false" diagonalDown="false">
@@ -670,16 +676,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </left>
       <right style="thin">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </right>
       <top style="thin">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </bottom>
       <diagonal/>
     </border>
@@ -720,23 +726,23 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </left>
       <right style="medium">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </right>
       <top style="medium">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </top>
       <bottom style="medium">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </bottom>
       <diagonal/>
     </border>
@@ -757,16 +763,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="hair">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </left>
       <right style="hair">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </right>
       <top style="hair">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </top>
       <bottom style="hair">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </bottom>
       <diagonal/>
     </border>
@@ -793,7 +799,7 @@
         <color rgb="FFFFFAF7"/>
       </right>
       <top style="medium">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -824,7 +830,7 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thick">
-        <color rgb="FFC9A24B"/>
+        <color rgb="FFE0B84C"/>
       </left>
       <right/>
       <top/>
@@ -998,7 +1004,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1162,7 +1168,7 @@
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFFF1CC"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FFB00040"/>
@@ -1171,14 +1177,14 @@
       <rgbColor rgb="FF8A5A00"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFF0D5DF"/>
+      <rgbColor rgb="FFFDE0E8"/>
       <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FFC2185B"/>
       <rgbColor rgb="FFFFF3C4"/>
       <rgbColor rgb="FFE3F4E7"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF5A1236"/>
+      <rgbColor rgb="FFFF4FA3"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
@@ -1192,19 +1198,19 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFFFFAF7"/>
       <rgbColor rgb="FFF8EDE6"/>
-      <rgbColor rgb="FFFFF1CC"/>
-      <rgbColor rgb="FFFDE0E8"/>
+      <rgbColor rgb="FFFBE7A6"/>
+      <rgbColor rgb="FFFCE9F0"/>
       <rgbColor rgb="FFF4B6CC"/>
-      <rgbColor rgb="FFFCE9F0"/>
-      <rgbColor rgb="FFF3E3B6"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFF0D5DF"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFE0B84C"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF7A5266"/>
-      <rgbColor rgb="FFC9A24B"/>
+      <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -1245,11 +1251,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="c9a24b"/>
+              <a:srgbClr val="e0b84c"/>
             </a:solidFill>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="c9a24b"/>
+                <a:srgbClr val="e0b84c"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1477,11 +1483,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="50455225"/>
-        <c:axId val="11777598"/>
+        <c:axId val="17324352"/>
+        <c:axId val="3282832"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50455225"/>
+        <c:axId val="17324352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1513,7 +1519,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11777598"/>
+        <c:crossAx val="3282832"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1521,7 +1527,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11777598"/>
+        <c:axId val="3282832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1563,7 +1569,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50455225"/>
+        <c:crossAx val="17324352"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1870,7 +1876,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF5A1236"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L34"/>
@@ -2823,7 +2829,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC9A24B"/>
+    <tabColor rgb="FFE0B84C"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:J37"/>
@@ -3796,7 +3802,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF5A1236"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:N36"/>

</xml_diff>

<commit_message>
Calculadora do celular e planilha no visual do site (topo vinho, titulo, botoes 3D, brilhos)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -374,7 +374,7 @@
     <font>
       <b val="true"/>
       <sz val="13"/>
-      <color rgb="FFFBE7A6"/>
+      <color rgb="FFF6D27A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -382,7 +382,7 @@
     <font>
       <i val="true"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFFFD3E8"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -598,7 +598,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -621,6 +621,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFAF7"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE91E78"/>
+        <bgColor rgb="FFC2185B"/>
       </patternFill>
     </fill>
     <fill>
@@ -662,7 +668,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE0B84C"/>
-        <bgColor rgb="FFFF9900"/>
+        <bgColor rgb="FFF6D27A"/>
       </patternFill>
     </fill>
   </fills>
@@ -863,7 +869,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -896,187 +902,191 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="11" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="11" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="23" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="12" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="8" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="8" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="6" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="29" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="11" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="10" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="10" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="23" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="23" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="6" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="20" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="5" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="28" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="28" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="29" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="10" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1177,7 +1187,7 @@
       <rgbColor rgb="FF8A5A00"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFFDE0E8"/>
+      <rgbColor rgb="FFF0D5DF"/>
       <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FFC2185B"/>
@@ -1189,7 +1199,7 @@
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFCE9F0"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
@@ -1199,10 +1209,10 @@
       <rgbColor rgb="FFFFFAF7"/>
       <rgbColor rgb="FFF8EDE6"/>
       <rgbColor rgb="FFFBE7A6"/>
-      <rgbColor rgb="FFFCE9F0"/>
+      <rgbColor rgb="FFFDE0E8"/>
       <rgbColor rgb="FFF4B6CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF0D5DF"/>
+      <rgbColor rgb="FFFFD3E8"/>
+      <rgbColor rgb="FFF6D27A"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1483,11 +1493,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="17324352"/>
-        <c:axId val="3282832"/>
+        <c:axId val="84900429"/>
+        <c:axId val="44734294"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="17324352"/>
+        <c:axId val="84900429"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1519,7 +1529,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3282832"/>
+        <c:crossAx val="44734294"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1527,7 +1537,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3282832"/>
+        <c:axId val="44734294"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1569,7 +1579,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17324352"/>
+        <c:crossAx val="84900429"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4476,12 +4486,12 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
     </row>
     <row r="2" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5"/>
@@ -4491,10 +4501,10 @@
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6"/>
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="52" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="51"/>
+      <c r="C3" s="52"/>
       <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4505,21 +4515,21 @@
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6"/>
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="53" t="s">
+      <c r="C5" s="54" t="s">
         <v>98</v>
       </c>
       <c r="D5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
-      <c r="B6" s="54" t="str">
+      <c r="B6" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B5="","",'Meus serviços'!A5)</f>
         <v>Esmaltação simples (mão)</v>
       </c>
-      <c r="C6" s="55" t="n">
+      <c r="C6" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B5="","",IF('Meus serviços'!D5&gt;='Meus serviços'!E5,'Meus serviços'!D5,'Meus serviços'!E5))</f>
         <v>36</v>
       </c>
@@ -4527,11 +4537,11 @@
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
-      <c r="B7" s="54" t="str">
+      <c r="B7" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B6="","",'Meus serviços'!A6)</f>
         <v>Esmaltação simples (pé)</v>
       </c>
-      <c r="C7" s="55" t="n">
+      <c r="C7" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B6="","",IF('Meus serviços'!D6&gt;='Meus serviços'!E6,'Meus serviços'!D6,'Meus serviços'!E6))</f>
         <v>40</v>
       </c>
@@ -4539,11 +4549,11 @@
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6"/>
-      <c r="B8" s="54" t="str">
+      <c r="B8" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B7="","",'Meus serviços'!A7)</f>
         <v>Mão + pé</v>
       </c>
-      <c r="C8" s="55" t="n">
+      <c r="C8" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B7="","",IF('Meus serviços'!D7&gt;='Meus serviços'!E7,'Meus serviços'!D7,'Meus serviços'!E7))</f>
         <v>72</v>
       </c>
@@ -4551,11 +4561,11 @@
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
-      <c r="B9" s="54" t="str">
+      <c r="B9" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B8="","",'Meus serviços'!A8)</f>
         <v>Esmaltação em gel (mão)</v>
       </c>
-      <c r="C9" s="55" t="n">
+      <c r="C9" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B8="","",IF('Meus serviços'!D8&gt;='Meus serviços'!E8,'Meus serviços'!D8,'Meus serviços'!E8))</f>
         <v>70</v>
       </c>
@@ -4563,11 +4573,11 @@
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6"/>
-      <c r="B10" s="54" t="str">
+      <c r="B10" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B9="","",'Meus serviços'!A9)</f>
         <v>Blindagem</v>
       </c>
-      <c r="C10" s="55" t="n">
+      <c r="C10" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B9="","",IF('Meus serviços'!D9&gt;='Meus serviços'!E9,'Meus serviços'!D9,'Meus serviços'!E9))</f>
         <v>90</v>
       </c>
@@ -4575,11 +4585,11 @@
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
-      <c r="B11" s="54" t="str">
+      <c r="B11" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B10="","",'Meus serviços'!A10)</f>
         <v>Alongamento em gel</v>
       </c>
-      <c r="C11" s="55" t="n">
+      <c r="C11" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B10="","",IF('Meus serviços'!D10&gt;='Meus serviços'!E10,'Meus serviços'!D10,'Meus serviços'!E10))</f>
         <v>180</v>
       </c>
@@ -4587,11 +4597,11 @@
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
-      <c r="B12" s="54" t="str">
+      <c r="B12" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B11="","",'Meus serviços'!A11)</f>
         <v>Manutenção de alongamento</v>
       </c>
-      <c r="C12" s="55" t="n">
+      <c r="C12" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B11="","",IF('Meus serviços'!D11&gt;='Meus serviços'!E11,'Meus serviços'!D11,'Meus serviços'!E11))</f>
         <v>120</v>
       </c>
@@ -4599,11 +4609,11 @@
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6"/>
-      <c r="B13" s="54" t="str">
+      <c r="B13" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B12="","",'Meus serviços'!A12)</f>
         <v>Remoção</v>
       </c>
-      <c r="C13" s="55" t="n">
+      <c r="C13" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B12="","",IF('Meus serviços'!D12&gt;='Meus serviços'!E12,'Meus serviços'!D12,'Meus serviços'!E12))</f>
         <v>25</v>
       </c>
@@ -4611,11 +4621,11 @@
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
-      <c r="B14" s="54" t="str">
+      <c r="B14" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B13="","",'Meus serviços'!A13)</f>
         <v/>
       </c>
-      <c r="C14" s="55" t="str">
+      <c r="C14" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B13="","",IF('Meus serviços'!D13&gt;='Meus serviços'!E13,'Meus serviços'!D13,'Meus serviços'!E13))</f>
         <v/>
       </c>
@@ -4623,11 +4633,11 @@
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
-      <c r="B15" s="54" t="str">
+      <c r="B15" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B14="","",'Meus serviços'!A14)</f>
         <v/>
       </c>
-      <c r="C15" s="55" t="str">
+      <c r="C15" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B14="","",IF('Meus serviços'!D14&gt;='Meus serviços'!E14,'Meus serviços'!D14,'Meus serviços'!E14))</f>
         <v/>
       </c>
@@ -4635,11 +4645,11 @@
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6"/>
-      <c r="B16" s="54" t="str">
+      <c r="B16" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B15="","",'Meus serviços'!A15)</f>
         <v/>
       </c>
-      <c r="C16" s="55" t="str">
+      <c r="C16" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B15="","",IF('Meus serviços'!D15&gt;='Meus serviços'!E15,'Meus serviços'!D15,'Meus serviços'!E15))</f>
         <v/>
       </c>
@@ -4647,11 +4657,11 @@
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
-      <c r="B17" s="54" t="str">
+      <c r="B17" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B16="","",'Meus serviços'!A16)</f>
         <v/>
       </c>
-      <c r="C17" s="55" t="str">
+      <c r="C17" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B16="","",IF('Meus serviços'!D16&gt;='Meus serviços'!E16,'Meus serviços'!D16,'Meus serviços'!E16))</f>
         <v/>
       </c>
@@ -4659,11 +4669,11 @@
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
-      <c r="B18" s="54" t="str">
+      <c r="B18" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B17="","",'Meus serviços'!A17)</f>
         <v/>
       </c>
-      <c r="C18" s="55" t="str">
+      <c r="C18" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B17="","",IF('Meus serviços'!D17&gt;='Meus serviços'!E17,'Meus serviços'!D17,'Meus serviços'!E17))</f>
         <v/>
       </c>
@@ -4671,11 +4681,11 @@
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6"/>
-      <c r="B19" s="54" t="str">
+      <c r="B19" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B18="","",'Meus serviços'!A18)</f>
         <v/>
       </c>
-      <c r="C19" s="55" t="str">
+      <c r="C19" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B18="","",IF('Meus serviços'!D18&gt;='Meus serviços'!E18,'Meus serviços'!D18,'Meus serviços'!E18))</f>
         <v/>
       </c>
@@ -4683,11 +4693,11 @@
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
-      <c r="B20" s="54" t="str">
+      <c r="B20" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B19="","",'Meus serviços'!A19)</f>
         <v/>
       </c>
-      <c r="C20" s="55" t="str">
+      <c r="C20" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B19="","",IF('Meus serviços'!D19&gt;='Meus serviços'!E19,'Meus serviços'!D19,'Meus serviços'!E19))</f>
         <v/>
       </c>
@@ -4695,11 +4705,11 @@
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6"/>
-      <c r="B21" s="54" t="str">
+      <c r="B21" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B20="","",'Meus serviços'!A20)</f>
         <v/>
       </c>
-      <c r="C21" s="55" t="str">
+      <c r="C21" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B20="","",IF('Meus serviços'!D20&gt;='Meus serviços'!E20,'Meus serviços'!D20,'Meus serviços'!E20))</f>
         <v/>
       </c>
@@ -4707,11 +4717,11 @@
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6"/>
-      <c r="B22" s="54" t="str">
+      <c r="B22" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B21="","",'Meus serviços'!A21)</f>
         <v/>
       </c>
-      <c r="C22" s="55" t="str">
+      <c r="C22" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B21="","",IF('Meus serviços'!D21&gt;='Meus serviços'!E21,'Meus serviços'!D21,'Meus serviços'!E21))</f>
         <v/>
       </c>
@@ -4719,11 +4729,11 @@
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6"/>
-      <c r="B23" s="54" t="str">
+      <c r="B23" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B22="","",'Meus serviços'!A22)</f>
         <v/>
       </c>
-      <c r="C23" s="55" t="str">
+      <c r="C23" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B22="","",IF('Meus serviços'!D22&gt;='Meus serviços'!E22,'Meus serviços'!D22,'Meus serviços'!E22))</f>
         <v/>
       </c>
@@ -4731,11 +4741,11 @@
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6"/>
-      <c r="B24" s="54" t="str">
+      <c r="B24" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B23="","",'Meus serviços'!A23)</f>
         <v/>
       </c>
-      <c r="C24" s="55" t="str">
+      <c r="C24" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B23="","",IF('Meus serviços'!D23&gt;='Meus serviços'!E23,'Meus serviços'!D23,'Meus serviços'!E23))</f>
         <v/>
       </c>
@@ -4743,11 +4753,11 @@
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6"/>
-      <c r="B25" s="54" t="str">
+      <c r="B25" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B24="","",'Meus serviços'!A24)</f>
         <v/>
       </c>
-      <c r="C25" s="55" t="str">
+      <c r="C25" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B24="","",IF('Meus serviços'!D24&gt;='Meus serviços'!E24,'Meus serviços'!D24,'Meus serviços'!E24))</f>
         <v/>
       </c>
@@ -4755,11 +4765,11 @@
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6"/>
-      <c r="B26" s="54" t="str">
+      <c r="B26" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B25="","",'Meus serviços'!A25)</f>
         <v/>
       </c>
-      <c r="C26" s="55" t="str">
+      <c r="C26" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B25="","",IF('Meus serviços'!D25&gt;='Meus serviços'!E25,'Meus serviços'!D25,'Meus serviços'!E25))</f>
         <v/>
       </c>
@@ -4767,11 +4777,11 @@
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6"/>
-      <c r="B27" s="54" t="str">
+      <c r="B27" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B26="","",'Meus serviços'!A26)</f>
         <v/>
       </c>
-      <c r="C27" s="55" t="str">
+      <c r="C27" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B26="","",IF('Meus serviços'!D26&gt;='Meus serviços'!E26,'Meus serviços'!D26,'Meus serviços'!E26))</f>
         <v/>
       </c>
@@ -4779,11 +4789,11 @@
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6"/>
-      <c r="B28" s="54" t="str">
+      <c r="B28" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B27="","",'Meus serviços'!A27)</f>
         <v/>
       </c>
-      <c r="C28" s="55" t="str">
+      <c r="C28" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B27="","",IF('Meus serviços'!D27&gt;='Meus serviços'!E27,'Meus serviços'!D27,'Meus serviços'!E27))</f>
         <v/>
       </c>
@@ -4791,11 +4801,11 @@
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6"/>
-      <c r="B29" s="54" t="str">
+      <c r="B29" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B28="","",'Meus serviços'!A28)</f>
         <v/>
       </c>
-      <c r="C29" s="55" t="str">
+      <c r="C29" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B28="","",IF('Meus serviços'!D28&gt;='Meus serviços'!E28,'Meus serviços'!D28,'Meus serviços'!E28))</f>
         <v/>
       </c>
@@ -4803,11 +4813,11 @@
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6"/>
-      <c r="B30" s="54" t="str">
+      <c r="B30" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B29="","",'Meus serviços'!A29)</f>
         <v/>
       </c>
-      <c r="C30" s="55" t="str">
+      <c r="C30" s="56" t="str">
         <f aca="false">IF('Meus serviços'!B29="","",IF('Meus serviços'!D29&gt;='Meus serviços'!E29,'Meus serviços'!D29,'Meus serviços'!E29))</f>
         <v/>
       </c>
@@ -4829,10 +4839,10 @@
     </row>
     <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6"/>
-      <c r="B33" s="56" t="s">
+      <c r="B33" s="57" t="s">
         <v>99</v>
       </c>
-      <c r="C33" s="56"/>
+      <c r="C33" s="57"/>
       <c r="D33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Planilha: titulos em fonte arredondada; hero: frase dourada no estilo da frase 'conta certa'
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -364,10 +364,9 @@
       <family val="0"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="28"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -388,18 +387,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="18"/>
       <color rgb="FF3A0A26"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="22"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -427,10 +424,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="14"/>
       <color rgb="FF3A0A26"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -465,10 +461,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="20"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -519,10 +514,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="18"/>
       <color rgb="FFC2185B"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -551,18 +545,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="26"/>
       <color rgb="FFC2185B"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="26"/>
       <color rgb="FFB00040"/>
-      <name val="Arial"/>
+      <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -1493,11 +1485,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="84900429"/>
-        <c:axId val="44734294"/>
+        <c:axId val="65278824"/>
+        <c:axId val="42548592"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="84900429"/>
+        <c:axId val="65278824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1529,7 +1521,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44734294"/>
+        <c:crossAx val="42548592"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1537,7 +1529,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44734294"/>
+        <c:axId val="42548592"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1579,7 +1571,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84900429"/>
+        <c:crossAx val="65278824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Tira referencias a unhas: icones, emojis, FAQ, exemplos variados na planilha, calculadora e imagens do site
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Kit Preço Certo</t>
   </si>
   <si>
-    <t xml:space="preserve">Calculadora de preço para manicure</t>
+    <t xml:space="preserve">Calculadora de preço para quem vende serviços</t>
   </si>
   <si>
     <t xml:space="preserve">Descubra quanto cobrar sem trabalhar no prejuízo.</t>
@@ -242,28 +242,28 @@
     <t xml:space="preserve">Lucro hoje (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Esmaltação simples (mão)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Esmaltação simples (pé)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mão + pé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Esmaltação em gel (mão)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blindagem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alongamento em gel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manutenção de alongamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remoção</t>
+    <t xml:space="preserve">Corte feminino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manicure (mão)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design de sobrancelha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limpeza de pele</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Massagem relaxante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extensão de cílios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depilação (perna)</t>
   </si>
   <si>
     <t xml:space="preserve">✦  Como o preço é calculado: (custo do tempo + material) ÷ (1 − taxa do cartão − margem), arredondado para cima ao real.</t>
@@ -1294,28 +1294,28 @@
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>Esmaltação simples (mão)</c:v>
+                  <c:v>Corte feminino</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Esmaltação simples (pé)</c:v>
+                  <c:v>Escova</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Mão + pé</c:v>
+                  <c:v>Manicure (mão)</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Esmaltação em gel (mão)</c:v>
+                  <c:v>Design de sobrancelha</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Blindagem</c:v>
+                  <c:v>Limpeza de pele</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Alongamento em gel</c:v>
+                  <c:v>Massagem relaxante</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Manutenção de alongamento</c:v>
+                  <c:v>Extensão de cílios</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Remoção</c:v>
+                  <c:v>Depilação (perna)</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v/>
@@ -1333,28 +1333,28 @@
                 <c:formatCode>"R$ "#,##0.00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>35</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>35</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>70</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>90</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>180</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>120</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>25</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1417,28 +1417,28 @@
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>Esmaltação simples (mão)</c:v>
+                  <c:v>Corte feminino</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Esmaltação simples (pé)</c:v>
+                  <c:v>Escova</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Mão + pé</c:v>
+                  <c:v>Manicure (mão)</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Esmaltação em gel (mão)</c:v>
+                  <c:v>Design de sobrancelha</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Blindagem</c:v>
+                  <c:v>Limpeza de pele</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Alongamento em gel</c:v>
+                  <c:v>Massagem relaxante</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Manutenção de alongamento</c:v>
+                  <c:v>Extensão de cílios</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Remoção</c:v>
+                  <c:v>Depilação (perna)</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v/>
@@ -1456,28 +1456,28 @@
                 <c:formatCode>"R$ "#,##0.00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>36</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>72</c:v>
-                </c:pt>
                 <c:pt idx="3">
-                  <c:v>66</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>84</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>145</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>109</c:v>
+                  <c:v>124</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>25</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1485,11 +1485,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="65278824"/>
-        <c:axId val="42548592"/>
+        <c:axId val="27821349"/>
+        <c:axId val="24487735"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65278824"/>
+        <c:axId val="27821349"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1521,7 +1521,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42548592"/>
+        <c:crossAx val="24487735"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1529,7 +1529,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42548592"/>
+        <c:axId val="24487735"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1571,7 +1571,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65278824"/>
+        <c:crossAx val="27821349"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2922,33 +2922,33 @@
         <v>72</v>
       </c>
       <c r="B5" s="38" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C5" s="39" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D5" s="39" t="n">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="E5" s="40" t="n">
         <f aca="false">IF(B5="","",ROUNDUP(H5/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="F5" s="41" t="str">
         <f aca="false">IF(OR(B5="",D5=""),"",IF(D5&gt;=E5,"OK: cobre custos e margem",IF(I5&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
-        <v>Atenção: pouca folga</v>
+        <v>OK: cobre custos e margem</v>
       </c>
       <c r="G5" s="42" t="n">
         <f aca="false">IF(B5="","",B5/60*'Meu custo por hora'!$B$25)</f>
-        <v>26.7143364718422</v>
+        <v>35.6191152957897</v>
       </c>
       <c r="H5" s="42" t="n">
         <f aca="false">IF(B5="","",G5+C5)</f>
-        <v>30.7143364718422</v>
+        <v>41.6191152957897</v>
       </c>
       <c r="I5" s="43" t="n">
         <f aca="false">IF(OR(B5="",D5=""),"",D5*(1-'Meu custo por hora'!$B$28)-H5)</f>
-        <v>2.88566352815776</v>
+        <v>35.1808847042103</v>
       </c>
       <c r="J5" s="6"/>
     </row>
@@ -2957,33 +2957,33 @@
         <v>73</v>
       </c>
       <c r="B6" s="38" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C6" s="39" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" s="39" t="n">
         <v>35</v>
       </c>
       <c r="E6" s="40" t="n">
         <f aca="false">IF(B6="","",ROUNDUP(H6/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F6" s="41" t="str">
         <f aca="false">IF(OR(B6="",D6=""),"",IF(D6&gt;=E6,"OK: cobre custos e margem",IF(I6&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
-        <v>PREJUÍZO: abaixo do custo</v>
+        <v>Atenção: pouca folga</v>
       </c>
       <c r="G6" s="42" t="n">
         <f aca="false">IF(B6="","",B6/60*'Meu custo por hora'!$B$25)</f>
-        <v>29.6825960798247</v>
+        <v>26.7143364718422</v>
       </c>
       <c r="H6" s="42" t="n">
         <f aca="false">IF(B6="","",G6+C6)</f>
-        <v>33.6825960798247</v>
+        <v>32.7143364718422</v>
       </c>
       <c r="I6" s="43" t="n">
         <f aca="false">IF(OR(B6="",D6=""),"",D6*(1-'Meu custo por hora'!$B$28)-H6)</f>
-        <v>-0.0825960798247181</v>
+        <v>0.885663528157757</v>
       </c>
       <c r="J6" s="6"/>
     </row>
@@ -2992,17 +2992,17 @@
         <v>74</v>
       </c>
       <c r="B7" s="38" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="C7" s="39" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D7" s="39" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E7" s="40" t="n">
         <f aca="false">IF(B7="","",ROUNDUP(H7/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="F7" s="41" t="str">
         <f aca="false">IF(OR(B7="",D7=""),"",IF(D7&gt;=E7,"OK: cobre custos e margem",IF(I7&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
@@ -3010,15 +3010,15 @@
       </c>
       <c r="G7" s="42" t="n">
         <f aca="false">IF(B7="","",B7/60*'Meu custo por hora'!$B$25)</f>
-        <v>53.4286729436845</v>
+        <v>26.7143364718422</v>
       </c>
       <c r="H7" s="42" t="n">
         <f aca="false">IF(B7="","",G7+C7)</f>
-        <v>61.4286729436845</v>
+        <v>30.7143364718422</v>
       </c>
       <c r="I7" s="43" t="n">
         <f aca="false">IF(OR(B7="",D7=""),"",D7*(1-'Meu custo por hora'!$B$28)-H7)</f>
-        <v>-3.8286729436845</v>
+        <v>-1.91433647184225</v>
       </c>
       <c r="J7" s="6"/>
     </row>
@@ -3027,17 +3027,17 @@
         <v>75</v>
       </c>
       <c r="B8" s="38" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="C8" s="39" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D8" s="39" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E8" s="40" t="n">
         <f aca="false">IF(B8="","",ROUNDUP(H8/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="F8" s="41" t="str">
         <f aca="false">IF(OR(B8="",D8=""),"",IF(D8&gt;=E8,"OK: cobre custos e margem",IF(I8&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
@@ -3045,15 +3045,15 @@
       </c>
       <c r="G8" s="42" t="n">
         <f aca="false">IF(B8="","",B8/60*'Meu custo por hora'!$B$25)</f>
-        <v>44.5238941197371</v>
+        <v>17.8095576478948</v>
       </c>
       <c r="H8" s="42" t="n">
         <f aca="false">IF(B8="","",G8+C8)</f>
-        <v>56.5238941197371</v>
+        <v>20.8095576478948</v>
       </c>
       <c r="I8" s="43" t="n">
         <f aca="false">IF(OR(B8="",D8=""),"",D8*(1-'Meu custo por hora'!$B$28)-H8)</f>
-        <v>10.6761058802629</v>
+        <v>17.5904423521052</v>
       </c>
       <c r="J8" s="6"/>
     </row>
@@ -3062,17 +3062,17 @@
         <v>76</v>
       </c>
       <c r="B9" s="38" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C9" s="39" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D9" s="39" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E9" s="40" t="n">
         <f aca="false">IF(B9="","",ROUNDUP(H9/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="F9" s="41" t="str">
         <f aca="false">IF(OR(B9="",D9=""),"",IF(D9&gt;=E9,"OK: cobre custos e margem",IF(I9&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
@@ -3080,15 +3080,15 @@
       </c>
       <c r="G9" s="42" t="n">
         <f aca="false">IF(B9="","",B9/60*'Meu custo por hora'!$B$25)</f>
-        <v>53.4286729436845</v>
+        <v>44.5238941197371</v>
       </c>
       <c r="H9" s="42" t="n">
         <f aca="false">IF(B9="","",G9+C9)</f>
-        <v>71.4286729436845</v>
+        <v>59.5238941197371</v>
       </c>
       <c r="I9" s="43" t="n">
         <f aca="false">IF(OR(B9="",D9=""),"",D9*(1-'Meu custo por hora'!$B$28)-H9)</f>
-        <v>14.9713270563155</v>
+        <v>55.6761058802629</v>
       </c>
       <c r="J9" s="6"/>
     </row>
@@ -3097,17 +3097,17 @@
         <v>77</v>
       </c>
       <c r="B10" s="38" t="n">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="C10" s="39" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="D10" s="39" t="n">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="E10" s="40" t="n">
         <f aca="false">IF(B10="","",ROUNDUP(H10/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>145</v>
+        <v>51</v>
       </c>
       <c r="F10" s="41" t="str">
         <f aca="false">IF(OR(B10="",D10=""),"",IF(D10&gt;=E10,"OK: cobre custos e margem",IF(I10&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
@@ -3115,15 +3115,15 @@
       </c>
       <c r="G10" s="42" t="n">
         <f aca="false">IF(B10="","",B10/60*'Meu custo por hora'!$B$25)</f>
-        <v>89.0477882394742</v>
+        <v>35.6191152957897</v>
       </c>
       <c r="H10" s="42" t="n">
         <f aca="false">IF(B10="","",G10+C10)</f>
-        <v>124.047788239474</v>
+        <v>43.6191152957897</v>
       </c>
       <c r="I10" s="43" t="n">
         <f aca="false">IF(OR(B10="",D10=""),"",D10*(1-'Meu custo por hora'!$B$28)-H10)</f>
-        <v>48.7522117605258</v>
+        <v>52.3808847042103</v>
       </c>
       <c r="J10" s="6"/>
     </row>
@@ -3135,14 +3135,14 @@
         <v>120</v>
       </c>
       <c r="C11" s="39" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D11" s="39" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="E11" s="40" t="n">
         <f aca="false">IF(B11="","",ROUNDUP(H11/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="F11" s="41" t="str">
         <f aca="false">IF(OR(B11="",D11=""),"",IF(D11&gt;=E11,"OK: cobre custos e margem",IF(I11&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
@@ -3154,11 +3154,11 @@
       </c>
       <c r="H11" s="42" t="n">
         <f aca="false">IF(B11="","",G11+C11)</f>
-        <v>93.2382305915793</v>
+        <v>106.238230591579</v>
       </c>
       <c r="I11" s="43" t="n">
         <f aca="false">IF(OR(B11="",D11=""),"",D11*(1-'Meu custo por hora'!$B$28)-H11)</f>
-        <v>21.9617694084207</v>
+        <v>66.5617694084207</v>
       </c>
       <c r="J11" s="6"/>
     </row>
@@ -3167,17 +3167,17 @@
         <v>79</v>
       </c>
       <c r="B12" s="38" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C12" s="39" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D12" s="39" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E12" s="40" t="n">
         <f aca="false">IF(B12="","",ROUNDUP(H12/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F12" s="41" t="str">
         <f aca="false">IF(OR(B12="",D12=""),"",IF(D12&gt;=E12,"OK: cobre custos e margem",IF(I12&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
@@ -3185,15 +3185,15 @@
       </c>
       <c r="G12" s="42" t="n">
         <f aca="false">IF(B12="","",B12/60*'Meu custo por hora'!$B$25)</f>
-        <v>17.8095576478948</v>
+        <v>23.7460768638598</v>
       </c>
       <c r="H12" s="42" t="n">
         <f aca="false">IF(B12="","",G12+C12)</f>
-        <v>20.8095576478948</v>
+        <v>31.7460768638598</v>
       </c>
       <c r="I12" s="43" t="n">
         <f aca="false">IF(OR(B12="",D12=""),"",D12*(1-'Meu custo por hora'!$B$28)-H12)</f>
-        <v>3.19044235210517</v>
+        <v>21.0539231361402</v>
       </c>
       <c r="J12" s="6"/>
     </row>
@@ -3923,13 +3923,13 @@
       <c r="G6" s="47"/>
       <c r="H6" s="47" t="n">
         <f aca="false">COUNTIF('Meus serviços'!F5:F29,"Atenção*")+COUNTIF('Meus serviços'!F5:F29,"PREJUÍZO*")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" s="47"/>
       <c r="J6" s="47"/>
       <c r="K6" s="48" t="n">
         <f aca="false">COUNTIF('Meus serviços'!F5:F29,"PREJUÍZO*")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" s="48"/>
       <c r="M6" s="48"/>
@@ -3979,7 +3979,7 @@
       <c r="A9" s="6"/>
       <c r="B9" s="50" t="str">
         <f aca="false">IF(K6&gt;0,"Atenção: "&amp;K6&amp;" serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.",IF(H6&gt;0,"Alguns serviços têm pouca folga. Compare o preço de hoje com o preço sugerido.","Os preços cadastrados cobrem seus custos e a margem. Revise quando seus gastos mudarem."))</f>
-        <v>Atenção: 2 serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.</v>
+        <v>Atenção: 1 serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.</v>
       </c>
       <c r="C9" s="50"/>
       <c r="D9" s="50"/>
@@ -4519,11 +4519,11 @@
       <c r="A6" s="6"/>
       <c r="B6" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B5="","",'Meus serviços'!A5)</f>
-        <v>Esmaltação simples (mão)</v>
+        <v>Corte feminino</v>
       </c>
       <c r="C6" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B5="","",IF('Meus serviços'!D5&gt;='Meus serviços'!E5,'Meus serviços'!D5,'Meus serviços'!E5))</f>
-        <v>36</v>
+        <v>80</v>
       </c>
       <c r="D6" s="6"/>
     </row>
@@ -4531,11 +4531,11 @@
       <c r="A7" s="6"/>
       <c r="B7" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B6="","",'Meus serviços'!A6)</f>
-        <v>Esmaltação simples (pé)</v>
+        <v>Escova</v>
       </c>
       <c r="C7" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B6="","",IF('Meus serviços'!D6&gt;='Meus serviços'!E6,'Meus serviços'!D6,'Meus serviços'!E6))</f>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D7" s="6"/>
     </row>
@@ -4543,11 +4543,11 @@
       <c r="A8" s="6"/>
       <c r="B8" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B7="","",'Meus serviços'!A7)</f>
-        <v>Mão + pé</v>
+        <v>Manicure (mão)</v>
       </c>
       <c r="C8" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B7="","",IF('Meus serviços'!D7&gt;='Meus serviços'!E7,'Meus serviços'!D7,'Meus serviços'!E7))</f>
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="D8" s="6"/>
     </row>
@@ -4555,11 +4555,11 @@
       <c r="A9" s="6"/>
       <c r="B9" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B8="","",'Meus serviços'!A8)</f>
-        <v>Esmaltação em gel (mão)</v>
+        <v>Design de sobrancelha</v>
       </c>
       <c r="C9" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B8="","",IF('Meus serviços'!D8&gt;='Meus serviços'!E8,'Meus serviços'!D8,'Meus serviços'!E8))</f>
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="D9" s="6"/>
     </row>
@@ -4567,11 +4567,11 @@
       <c r="A10" s="6"/>
       <c r="B10" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B9="","",'Meus serviços'!A9)</f>
-        <v>Blindagem</v>
+        <v>Limpeza de pele</v>
       </c>
       <c r="C10" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B9="","",IF('Meus serviços'!D9&gt;='Meus serviços'!E9,'Meus serviços'!D9,'Meus serviços'!E9))</f>
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D10" s="6"/>
     </row>
@@ -4579,11 +4579,11 @@
       <c r="A11" s="6"/>
       <c r="B11" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B10="","",'Meus serviços'!A10)</f>
-        <v>Alongamento em gel</v>
+        <v>Massagem relaxante</v>
       </c>
       <c r="C11" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B10="","",IF('Meus serviços'!D10&gt;='Meus serviços'!E10,'Meus serviços'!D10,'Meus serviços'!E10))</f>
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="D11" s="6"/>
     </row>
@@ -4591,11 +4591,11 @@
       <c r="A12" s="6"/>
       <c r="B12" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B11="","",'Meus serviços'!A11)</f>
-        <v>Manutenção de alongamento</v>
+        <v>Extensão de cílios</v>
       </c>
       <c r="C12" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B11="","",IF('Meus serviços'!D11&gt;='Meus serviços'!E11,'Meus serviços'!D11,'Meus serviços'!E11))</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="D12" s="6"/>
     </row>
@@ -4603,11 +4603,11 @@
       <c r="A13" s="6"/>
       <c r="B13" s="55" t="str">
         <f aca="false">IF('Meus serviços'!B12="","",'Meus serviços'!A12)</f>
-        <v>Remoção</v>
+        <v>Depilação (perna)</v>
       </c>
       <c r="C13" s="56" t="n">
         <f aca="false">IF('Meus serviços'!B12="","",IF('Meus serviços'!D12&gt;='Meus serviços'!E12,'Meus serviços'!D12,'Meus serviços'!E12))</f>
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="D13" s="6"/>
     </row>

</xml_diff>

<commit_message>
Planilha: logo nova e aba Meu Painel; site: abas Meu custo por hora/Meus servicos/Meu Painel com prints reais e troca automatica
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Leia primeiro" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Meu custo por hora" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Meus serviços" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Painel" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Meu Painel" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Tabela para divulgar" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -68,7 +68,7 @@
     <t xml:space="preserve">Ver painel  →</t>
   </si>
   <si>
-    <t xml:space="preserve">Você recebe o preço sugerido, o lucro de hoje e um aviso quando um serviço está dando prejuízo. Veja o resumo no “Painel” e copie a “Tabela para divulgar”.</t>
+    <t xml:space="preserve">Você recebe o preço sugerido, o lucro de hoje e um aviso quando um serviço está dando prejuízo. Veja o resumo no “Meu Painel” e copie a “Tabela para divulgar”.</t>
   </si>
   <si>
     <t xml:space="preserve">Como ler as cores</t>
@@ -1485,11 +1485,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="27821349"/>
-        <c:axId val="24487735"/>
+        <c:axId val="74484580"/>
+        <c:axId val="1970280"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27821349"/>
+        <c:axId val="74484580"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1521,7 +1521,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24487735"/>
+        <c:crossAx val="1970280"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1529,7 +1529,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24487735"/>
+        <c:axId val="1970280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1571,7 +1571,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27821349"/>
+        <c:crossAx val="74484580"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2460,7 +2460,7 @@
   <hyperlinks>
     <hyperlink ref="J10" location="'Meu custo por hora'!A1" display="Abrir aba  →"/>
     <hyperlink ref="J13" location="'Meus serviços'!A1" display="Abrir aba  →"/>
-    <hyperlink ref="J16" location="'Painel'!A1" display="Ver painel  →"/>
+    <hyperlink ref="J16" location="'Meu Painel'!A1" display="Ver painel  →"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Planilha mais profissional (logo, navegacao, indicadores extras, dicas nas celulas) e secao do bonus com notebook, selos e legendas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="111">
   <si>
     <t xml:space="preserve">Kit Preço Certo</t>
   </si>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Calculadora de preço para quem vende serviços</t>
   </si>
   <si>
-    <t xml:space="preserve">Descubra quanto cobrar sem trabalhar no prejuízo.</t>
+    <t xml:space="preserve">Fórmulas prontas: é só preencher as células amarelas. Não precisa saber Excel.</t>
   </si>
   <si>
     <t xml:space="preserve">Comece em 3 passos</t>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Passo 1  ·  Quanto custa a sua hora</t>
   </si>
   <si>
-    <t xml:space="preserve">Preencha só as células amarelas. Os valores já preenchidos são exemplos: troque pelos seus.</t>
+    <t xml:space="preserve">Preencha só as células amarelas. As contas já estão prontas. Os valores preenchidos são exemplos: troque pelos seus.</t>
   </si>
   <si>
     <t xml:space="preserve">Gastos fixos do mês (R$)</t>
@@ -209,10 +209,16 @@
     <t xml:space="preserve">Para imprevistos e crescer. 0% se não quiser</t>
   </si>
   <si>
+    <t xml:space="preserve">Pronto! Próximo passo: cadastrar seus serviços  →</t>
+  </si>
+  <si>
     <t xml:space="preserve">Passo 2  ·  Preço sugerido por serviço</t>
   </si>
   <si>
-    <t xml:space="preserve">Preencha as células amarelas (A a D). O PREÇO SUGERIDO aparece logo ao lado. Os serviços abaixo são EXEMPLOS: troque pelos seus.</t>
+    <t xml:space="preserve">Próximo: Meu Painel  →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preencha as células amarelas (A a D). O PREÇO SUGERIDO aparece sozinho ao lado. Os serviços abaixo são EXEMPLOS: troque pelos seus.</t>
   </si>
   <si>
     <t xml:space="preserve">Serviço</t>
@@ -281,7 +287,10 @@
     <t xml:space="preserve">Seu painel de preços</t>
   </si>
   <si>
-    <t xml:space="preserve">Resumo automático feito com o que você preencheu nas abas anteriores.</t>
+    <t xml:space="preserve">Ver Tabela para divulgar  →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumo automático feito com o que você preencheu nas abas anteriores. Aqui você não digita nada.</t>
   </si>
   <si>
     <t xml:space="preserve">CUSTO DA SUA HORA</t>
@@ -306,6 +315,30 @@
   </si>
   <si>
     <t xml:space="preserve">preço abaixo do custo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERVIÇOS OK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUCRO MÉDIO HOJE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAIS LUCRATIVO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEDE MAIS ATENÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cobrem custos e margem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">por atendimento, após a maquininha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maior lucro por atendimento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">menor lucro por atendimento</t>
   </si>
   <si>
     <t xml:space="preserve">Quanto você cobra hoje × preço sugerido</t>
@@ -330,7 +363,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;R$ &quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
@@ -338,9 +371,10 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
     <numFmt numFmtId="170" formatCode="&quot;R$ &quot;#,##0.00;[RED]&quot;-R$ &quot;#,##0.00"/>
-    <numFmt numFmtId="171" formatCode="&quot;R$ &quot;#,##0"/>
+    <numFmt numFmtId="171" formatCode="@"/>
+    <numFmt numFmtId="172" formatCode="&quot;R$ &quot;#,##0"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,7 +414,7 @@
     </font>
     <font>
       <i val="true"/>
-      <sz val="11"/>
+      <sz val="10.5"/>
       <color rgb="FFFFD3E8"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -522,6 +556,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF3A0A26"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
@@ -553,6 +595,34 @@
     </font>
     <font>
       <sz val="26"/>
+      <color rgb="FFB00040"/>
+      <name val="Arial Rounded MT Bold"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="26"/>
+      <color rgb="FF1B6B3A"/>
+      <name val="Arial Rounded MT Bold"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color rgb="FFC2185B"/>
+      <name val="Arial Rounded MT Bold"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF1B6B3A"/>
+      <name val="Arial Rounded MT Bold"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color rgb="FFB00040"/>
       <name val="Arial Rounded MT Bold"/>
       <family val="0"/>
@@ -861,7 +931,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="63">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -939,7 +1009,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="7" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -998,7 +1068,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1022,7 +1096,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="27" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1042,15 +1116,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="6" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="6" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="29" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1058,10 +1128,30 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="30" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="21" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="31" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="32" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="33" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="34" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="19" fillId="11" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1070,7 +1160,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="36" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1086,11 +1176,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="32" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="37" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="38" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1485,11 +1575,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="74484580"/>
-        <c:axId val="1970280"/>
+        <c:axId val="25424270"/>
+        <c:axId val="80355751"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74484580"/>
+        <c:axId val="25424270"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1521,7 +1611,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1970280"/>
+        <c:crossAx val="80355751"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1529,7 +1619,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1970280"/>
+        <c:axId val="80355751"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1571,7 +1661,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74484580"/>
+        <c:crossAx val="25424270"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1669,24 +1759,108 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>114480</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>552240</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>533160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="114480" y="95400"/>
+          <a:ext cx="437760" cy="437760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>114480</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>552240</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>533160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="114480" y="95400"/>
+          <a:ext cx="437760" cy="437760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>415440</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>26640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="1" name="Chart 1"/>
+        <xdr:cNvPr id="3" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="211320" y="3305160"/>
+        <a:off x="211320" y="4762440"/>
         <a:ext cx="9719640" cy="3455640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1695,6 +1869,43 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>114480</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>340920</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>533160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="114480" y="95400"/>
+          <a:ext cx="437760" cy="437760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2479,7 +2690,7 @@
     <tabColor rgb="FFE91E78"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -2488,13 +2699,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
         <v>28</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
@@ -2773,10 +2984,12 @@
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
+    <row r="31" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
       <c r="D31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2785,9 +2998,15 @@
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
     </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:D1"/>
+  <mergeCells count="9">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:C4"/>
@@ -2795,8 +3014,9 @@
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A31:C31"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation allowBlank="false" error="Digite um valor entre 0.5 e 24 (porcentagem: ex. 65%)." errorStyle="stop" errorTitle="Valor fora do esperado" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B18" type="decimal">
       <formula1>0.5</formula1>
       <formula2>24</formula2>
@@ -2817,7 +3037,18 @@
       <formula1>0</formula1>
       <formula2>0.5</formula2>
     </dataValidation>
+    <dataValidation allowBlank="true" error="Digite um valor em reais (ex.: 150)." errorStyle="stop" errorTitle="Valor em reais" operator="greaterThanOrEqual" prompt="Digite quanto você gasta por mês com isso, em reais. Se não tem esse gasto, ponha 0." promptTitle="Gasto do mês" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B5:B11" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Digite um valor em reais (ex.: 3000)." errorStyle="stop" errorTitle="Valor em reais" operator="greaterThanOrEqual" prompt="Quanto você quer tirar para você por mês, além dos gastos." promptTitle="Seu salário" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B15" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A31" location="'Meus serviços'!A1" display="Pronto! Próximo passo: cadastrar seus serviços  →"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2825,6 +3056,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2847,23 +3079,25 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
       <c r="E1" s="19"/>
       <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
+      <c r="G1" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -2888,769 +3122,769 @@
       <c r="J3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="34" t="s">
+      <c r="A4" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="B4" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="C4" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="D4" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="36" t="s">
+      <c r="E4" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="36" t="s">
+      <c r="F4" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="G4" s="37" t="s">
         <v>71</v>
       </c>
+      <c r="H4" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="I4" s="37" t="s">
+        <v>73</v>
+      </c>
       <c r="J4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="38" t="n">
+      <c r="A5" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C5" s="39" t="n">
+      <c r="C5" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="39" t="n">
+      <c r="D5" s="40" t="n">
         <v>80</v>
       </c>
-      <c r="E5" s="40" t="n">
+      <c r="E5" s="41" t="n">
         <f aca="false">IF(B5="","",ROUNDUP(H5/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>49</v>
       </c>
-      <c r="F5" s="41" t="str">
+      <c r="F5" s="42" t="str">
         <f aca="false">IF(OR(B5="",D5=""),"",IF(D5&gt;=E5,"OK: cobre custos e margem",IF(I5&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>OK: cobre custos e margem</v>
       </c>
-      <c r="G5" s="42" t="n">
+      <c r="G5" s="43" t="n">
         <f aca="false">IF(B5="","",B5/60*'Meu custo por hora'!$B$25)</f>
         <v>35.6191152957897</v>
       </c>
-      <c r="H5" s="42" t="n">
+      <c r="H5" s="43" t="n">
         <f aca="false">IF(B5="","",G5+C5)</f>
         <v>41.6191152957897</v>
       </c>
-      <c r="I5" s="43" t="n">
+      <c r="I5" s="44" t="n">
         <f aca="false">IF(OR(B5="",D5=""),"",D5*(1-'Meu custo por hora'!$B$28)-H5)</f>
         <v>35.1808847042103</v>
       </c>
       <c r="J5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="38" t="n">
+      <c r="A6" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="39" t="n">
         <v>45</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="C6" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="39" t="n">
+      <c r="D6" s="40" t="n">
         <v>35</v>
       </c>
-      <c r="E6" s="40" t="n">
+      <c r="E6" s="41" t="n">
         <f aca="false">IF(B6="","",ROUNDUP(H6/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>39</v>
       </c>
-      <c r="F6" s="41" t="str">
+      <c r="F6" s="42" t="str">
         <f aca="false">IF(OR(B6="",D6=""),"",IF(D6&gt;=E6,"OK: cobre custos e margem",IF(I6&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>Atenção: pouca folga</v>
       </c>
-      <c r="G6" s="42" t="n">
+      <c r="G6" s="43" t="n">
         <f aca="false">IF(B6="","",B6/60*'Meu custo por hora'!$B$25)</f>
         <v>26.7143364718422</v>
       </c>
-      <c r="H6" s="42" t="n">
+      <c r="H6" s="43" t="n">
         <f aca="false">IF(B6="","",G6+C6)</f>
         <v>32.7143364718422</v>
       </c>
-      <c r="I6" s="43" t="n">
+      <c r="I6" s="44" t="n">
         <f aca="false">IF(OR(B6="",D6=""),"",D6*(1-'Meu custo por hora'!$B$28)-H6)</f>
         <v>0.885663528157757</v>
       </c>
       <c r="J6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="38" t="n">
+      <c r="A7" s="38" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="39" t="n">
         <v>45</v>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="C7" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="39" t="n">
+      <c r="D7" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E7" s="41" t="n">
         <f aca="false">IF(B7="","",ROUNDUP(H7/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>36</v>
       </c>
-      <c r="F7" s="41" t="str">
+      <c r="F7" s="42" t="str">
         <f aca="false">IF(OR(B7="",D7=""),"",IF(D7&gt;=E7,"OK: cobre custos e margem",IF(I7&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>PREJUÍZO: abaixo do custo</v>
       </c>
-      <c r="G7" s="42" t="n">
+      <c r="G7" s="43" t="n">
         <f aca="false">IF(B7="","",B7/60*'Meu custo por hora'!$B$25)</f>
         <v>26.7143364718422</v>
       </c>
-      <c r="H7" s="42" t="n">
+      <c r="H7" s="43" t="n">
         <f aca="false">IF(B7="","",G7+C7)</f>
         <v>30.7143364718422</v>
       </c>
-      <c r="I7" s="43" t="n">
+      <c r="I7" s="44" t="n">
         <f aca="false">IF(OR(B7="",D7=""),"",D7*(1-'Meu custo por hora'!$B$28)-H7)</f>
         <v>-1.91433647184225</v>
       </c>
       <c r="J7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="38" t="n">
+      <c r="A8" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="39" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="C8" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="39" t="n">
+      <c r="D8" s="40" t="n">
         <v>40</v>
       </c>
-      <c r="E8" s="40" t="n">
+      <c r="E8" s="41" t="n">
         <f aca="false">IF(B8="","",ROUNDUP(H8/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>25</v>
       </c>
-      <c r="F8" s="41" t="str">
+      <c r="F8" s="42" t="str">
         <f aca="false">IF(OR(B8="",D8=""),"",IF(D8&gt;=E8,"OK: cobre custos e margem",IF(I8&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>OK: cobre custos e margem</v>
       </c>
-      <c r="G8" s="42" t="n">
+      <c r="G8" s="43" t="n">
         <f aca="false">IF(B8="","",B8/60*'Meu custo por hora'!$B$25)</f>
         <v>17.8095576478948</v>
       </c>
-      <c r="H8" s="42" t="n">
+      <c r="H8" s="43" t="n">
         <f aca="false">IF(B8="","",G8+C8)</f>
         <v>20.8095576478948</v>
       </c>
-      <c r="I8" s="43" t="n">
+      <c r="I8" s="44" t="n">
         <f aca="false">IF(OR(B8="",D8=""),"",D8*(1-'Meu custo por hora'!$B$28)-H8)</f>
         <v>17.5904423521052</v>
       </c>
       <c r="J8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="38" t="n">
+      <c r="A9" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="39" t="n">
         <v>75</v>
       </c>
-      <c r="C9" s="39" t="n">
+      <c r="C9" s="40" t="n">
         <v>15</v>
       </c>
-      <c r="D9" s="39" t="n">
+      <c r="D9" s="40" t="n">
         <v>120</v>
       </c>
-      <c r="E9" s="40" t="n">
+      <c r="E9" s="41" t="n">
         <f aca="false">IF(B9="","",ROUNDUP(H9/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>70</v>
       </c>
-      <c r="F9" s="41" t="str">
+      <c r="F9" s="42" t="str">
         <f aca="false">IF(OR(B9="",D9=""),"",IF(D9&gt;=E9,"OK: cobre custos e margem",IF(I9&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>OK: cobre custos e margem</v>
       </c>
-      <c r="G9" s="42" t="n">
+      <c r="G9" s="43" t="n">
         <f aca="false">IF(B9="","",B9/60*'Meu custo por hora'!$B$25)</f>
         <v>44.5238941197371</v>
       </c>
-      <c r="H9" s="42" t="n">
+      <c r="H9" s="43" t="n">
         <f aca="false">IF(B9="","",G9+C9)</f>
         <v>59.5238941197371</v>
       </c>
-      <c r="I9" s="43" t="n">
+      <c r="I9" s="44" t="n">
         <f aca="false">IF(OR(B9="",D9=""),"",D9*(1-'Meu custo por hora'!$B$28)-H9)</f>
         <v>55.6761058802629</v>
       </c>
       <c r="J9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" s="38" t="n">
+      <c r="A10" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="39" t="n">
         <v>60</v>
       </c>
-      <c r="C10" s="39" t="n">
+      <c r="C10" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="39" t="n">
+      <c r="D10" s="40" t="n">
         <v>100</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="E10" s="41" t="n">
         <f aca="false">IF(B10="","",ROUNDUP(H10/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>51</v>
       </c>
-      <c r="F10" s="41" t="str">
+      <c r="F10" s="42" t="str">
         <f aca="false">IF(OR(B10="",D10=""),"",IF(D10&gt;=E10,"OK: cobre custos e margem",IF(I10&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>OK: cobre custos e margem</v>
       </c>
-      <c r="G10" s="42" t="n">
+      <c r="G10" s="43" t="n">
         <f aca="false">IF(B10="","",B10/60*'Meu custo por hora'!$B$25)</f>
         <v>35.6191152957897</v>
       </c>
-      <c r="H10" s="42" t="n">
+      <c r="H10" s="43" t="n">
         <f aca="false">IF(B10="","",G10+C10)</f>
         <v>43.6191152957897</v>
       </c>
-      <c r="I10" s="43" t="n">
+      <c r="I10" s="44" t="n">
         <f aca="false">IF(OR(B10="",D10=""),"",D10*(1-'Meu custo por hora'!$B$28)-H10)</f>
         <v>52.3808847042103</v>
       </c>
       <c r="J10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="38" t="n">
+      <c r="A11" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="39" t="n">
         <v>120</v>
       </c>
-      <c r="C11" s="39" t="n">
+      <c r="C11" s="40" t="n">
         <v>35</v>
       </c>
-      <c r="D11" s="39" t="n">
+      <c r="D11" s="40" t="n">
         <v>180</v>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="E11" s="41" t="n">
         <f aca="false">IF(B11="","",ROUNDUP(H11/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>124</v>
       </c>
-      <c r="F11" s="41" t="str">
+      <c r="F11" s="42" t="str">
         <f aca="false">IF(OR(B11="",D11=""),"",IF(D11&gt;=E11,"OK: cobre custos e margem",IF(I11&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>OK: cobre custos e margem</v>
       </c>
-      <c r="G11" s="42" t="n">
+      <c r="G11" s="43" t="n">
         <f aca="false">IF(B11="","",B11/60*'Meu custo por hora'!$B$25)</f>
         <v>71.2382305915793</v>
       </c>
-      <c r="H11" s="42" t="n">
+      <c r="H11" s="43" t="n">
         <f aca="false">IF(B11="","",G11+C11)</f>
         <v>106.238230591579</v>
       </c>
-      <c r="I11" s="43" t="n">
+      <c r="I11" s="44" t="n">
         <f aca="false">IF(OR(B11="",D11=""),"",D11*(1-'Meu custo por hora'!$B$28)-H11)</f>
         <v>66.5617694084207</v>
       </c>
       <c r="J11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="38" t="n">
+      <c r="A12" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="39" t="n">
         <v>40</v>
       </c>
-      <c r="C12" s="39" t="n">
+      <c r="C12" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="D12" s="39" t="n">
+      <c r="D12" s="40" t="n">
         <v>55</v>
       </c>
-      <c r="E12" s="40" t="n">
+      <c r="E12" s="41" t="n">
         <f aca="false">IF(B12="","",ROUNDUP(H12/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v>37</v>
       </c>
-      <c r="F12" s="41" t="str">
+      <c r="F12" s="42" t="str">
         <f aca="false">IF(OR(B12="",D12=""),"",IF(D12&gt;=E12,"OK: cobre custos e margem",IF(I12&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v>OK: cobre custos e margem</v>
       </c>
-      <c r="G12" s="42" t="n">
+      <c r="G12" s="43" t="n">
         <f aca="false">IF(B12="","",B12/60*'Meu custo por hora'!$B$25)</f>
         <v>23.7460768638598</v>
       </c>
-      <c r="H12" s="42" t="n">
+      <c r="H12" s="43" t="n">
         <f aca="false">IF(B12="","",G12+C12)</f>
         <v>31.7460768638598</v>
       </c>
-      <c r="I12" s="43" t="n">
+      <c r="I12" s="44" t="n">
         <f aca="false">IF(OR(B12="",D12=""),"",D12*(1-'Meu custo por hora'!$B$28)-H12)</f>
         <v>21.0539231361402</v>
       </c>
       <c r="J12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="40" t="str">
+      <c r="A13" s="38"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="40"/>
+      <c r="E13" s="41" t="str">
         <f aca="false">IF(B13="","",ROUNDUP(H13/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F13" s="41" t="str">
+      <c r="F13" s="42" t="str">
         <f aca="false">IF(OR(B13="",D13=""),"",IF(D13&gt;=E13,"OK: cobre custos e margem",IF(I13&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G13" s="42" t="str">
+      <c r="G13" s="43" t="str">
         <f aca="false">IF(B13="","",B13/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H13" s="42" t="str">
+      <c r="H13" s="43" t="str">
         <f aca="false">IF(B13="","",G13+C13)</f>
         <v/>
       </c>
-      <c r="I13" s="43" t="str">
+      <c r="I13" s="44" t="str">
         <f aca="false">IF(OR(B13="",D13=""),"",D13*(1-'Meu custo por hora'!$B$28)-H13)</f>
         <v/>
       </c>
       <c r="J13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="40" t="str">
+      <c r="A14" s="38"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="41" t="str">
         <f aca="false">IF(B14="","",ROUNDUP(H14/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F14" s="41" t="str">
+      <c r="F14" s="42" t="str">
         <f aca="false">IF(OR(B14="",D14=""),"",IF(D14&gt;=E14,"OK: cobre custos e margem",IF(I14&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G14" s="42" t="str">
+      <c r="G14" s="43" t="str">
         <f aca="false">IF(B14="","",B14/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H14" s="42" t="str">
+      <c r="H14" s="43" t="str">
         <f aca="false">IF(B14="","",G14+C14)</f>
         <v/>
       </c>
-      <c r="I14" s="43" t="str">
+      <c r="I14" s="44" t="str">
         <f aca="false">IF(OR(B14="",D14=""),"",D14*(1-'Meu custo por hora'!$B$28)-H14)</f>
         <v/>
       </c>
       <c r="J14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40" t="str">
+      <c r="A15" s="38"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="41" t="str">
         <f aca="false">IF(B15="","",ROUNDUP(H15/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F15" s="41" t="str">
+      <c r="F15" s="42" t="str">
         <f aca="false">IF(OR(B15="",D15=""),"",IF(D15&gt;=E15,"OK: cobre custos e margem",IF(I15&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G15" s="42" t="str">
+      <c r="G15" s="43" t="str">
         <f aca="false">IF(B15="","",B15/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H15" s="42" t="str">
+      <c r="H15" s="43" t="str">
         <f aca="false">IF(B15="","",G15+C15)</f>
         <v/>
       </c>
-      <c r="I15" s="43" t="str">
+      <c r="I15" s="44" t="str">
         <f aca="false">IF(OR(B15="",D15=""),"",D15*(1-'Meu custo por hora'!$B$28)-H15)</f>
         <v/>
       </c>
       <c r="J15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="40" t="str">
+      <c r="A16" s="38"/>
+      <c r="B16" s="39"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="41" t="str">
         <f aca="false">IF(B16="","",ROUNDUP(H16/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F16" s="41" t="str">
+      <c r="F16" s="42" t="str">
         <f aca="false">IF(OR(B16="",D16=""),"",IF(D16&gt;=E16,"OK: cobre custos e margem",IF(I16&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G16" s="42" t="str">
+      <c r="G16" s="43" t="str">
         <f aca="false">IF(B16="","",B16/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H16" s="42" t="str">
+      <c r="H16" s="43" t="str">
         <f aca="false">IF(B16="","",G16+C16)</f>
         <v/>
       </c>
-      <c r="I16" s="43" t="str">
+      <c r="I16" s="44" t="str">
         <f aca="false">IF(OR(B16="",D16=""),"",D16*(1-'Meu custo por hora'!$B$28)-H16)</f>
         <v/>
       </c>
       <c r="J16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="40" t="str">
+      <c r="A17" s="38"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="41" t="str">
         <f aca="false">IF(B17="","",ROUNDUP(H17/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F17" s="41" t="str">
+      <c r="F17" s="42" t="str">
         <f aca="false">IF(OR(B17="",D17=""),"",IF(D17&gt;=E17,"OK: cobre custos e margem",IF(I17&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G17" s="42" t="str">
+      <c r="G17" s="43" t="str">
         <f aca="false">IF(B17="","",B17/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H17" s="42" t="str">
+      <c r="H17" s="43" t="str">
         <f aca="false">IF(B17="","",G17+C17)</f>
         <v/>
       </c>
-      <c r="I17" s="43" t="str">
+      <c r="I17" s="44" t="str">
         <f aca="false">IF(OR(B17="",D17=""),"",D17*(1-'Meu custo por hora'!$B$28)-H17)</f>
         <v/>
       </c>
       <c r="J17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="40" t="str">
+      <c r="A18" s="38"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="41" t="str">
         <f aca="false">IF(B18="","",ROUNDUP(H18/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F18" s="41" t="str">
+      <c r="F18" s="42" t="str">
         <f aca="false">IF(OR(B18="",D18=""),"",IF(D18&gt;=E18,"OK: cobre custos e margem",IF(I18&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G18" s="42" t="str">
+      <c r="G18" s="43" t="str">
         <f aca="false">IF(B18="","",B18/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H18" s="42" t="str">
+      <c r="H18" s="43" t="str">
         <f aca="false">IF(B18="","",G18+C18)</f>
         <v/>
       </c>
-      <c r="I18" s="43" t="str">
+      <c r="I18" s="44" t="str">
         <f aca="false">IF(OR(B18="",D18=""),"",D18*(1-'Meu custo por hora'!$B$28)-H18)</f>
         <v/>
       </c>
       <c r="J18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="40" t="str">
+      <c r="A19" s="38"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="41" t="str">
         <f aca="false">IF(B19="","",ROUNDUP(H19/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F19" s="41" t="str">
+      <c r="F19" s="42" t="str">
         <f aca="false">IF(OR(B19="",D19=""),"",IF(D19&gt;=E19,"OK: cobre custos e margem",IF(I19&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G19" s="42" t="str">
+      <c r="G19" s="43" t="str">
         <f aca="false">IF(B19="","",B19/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H19" s="42" t="str">
+      <c r="H19" s="43" t="str">
         <f aca="false">IF(B19="","",G19+C19)</f>
         <v/>
       </c>
-      <c r="I19" s="43" t="str">
+      <c r="I19" s="44" t="str">
         <f aca="false">IF(OR(B19="",D19=""),"",D19*(1-'Meu custo por hora'!$B$28)-H19)</f>
         <v/>
       </c>
       <c r="J19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="40" t="str">
+      <c r="A20" s="38"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="41" t="str">
         <f aca="false">IF(B20="","",ROUNDUP(H20/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F20" s="41" t="str">
+      <c r="F20" s="42" t="str">
         <f aca="false">IF(OR(B20="",D20=""),"",IF(D20&gt;=E20,"OK: cobre custos e margem",IF(I20&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G20" s="42" t="str">
+      <c r="G20" s="43" t="str">
         <f aca="false">IF(B20="","",B20/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H20" s="42" t="str">
+      <c r="H20" s="43" t="str">
         <f aca="false">IF(B20="","",G20+C20)</f>
         <v/>
       </c>
-      <c r="I20" s="43" t="str">
+      <c r="I20" s="44" t="str">
         <f aca="false">IF(OR(B20="",D20=""),"",D20*(1-'Meu custo por hora'!$B$28)-H20)</f>
         <v/>
       </c>
       <c r="J20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40" t="str">
+      <c r="A21" s="38"/>
+      <c r="B21" s="39"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="41" t="str">
         <f aca="false">IF(B21="","",ROUNDUP(H21/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F21" s="41" t="str">
+      <c r="F21" s="42" t="str">
         <f aca="false">IF(OR(B21="",D21=""),"",IF(D21&gt;=E21,"OK: cobre custos e margem",IF(I21&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G21" s="42" t="str">
+      <c r="G21" s="43" t="str">
         <f aca="false">IF(B21="","",B21/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H21" s="42" t="str">
+      <c r="H21" s="43" t="str">
         <f aca="false">IF(B21="","",G21+C21)</f>
         <v/>
       </c>
-      <c r="I21" s="43" t="str">
+      <c r="I21" s="44" t="str">
         <f aca="false">IF(OR(B21="",D21=""),"",D21*(1-'Meu custo por hora'!$B$28)-H21)</f>
         <v/>
       </c>
       <c r="J21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="40" t="str">
+      <c r="A22" s="38"/>
+      <c r="B22" s="39"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="41" t="str">
         <f aca="false">IF(B22="","",ROUNDUP(H22/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F22" s="41" t="str">
+      <c r="F22" s="42" t="str">
         <f aca="false">IF(OR(B22="",D22=""),"",IF(D22&gt;=E22,"OK: cobre custos e margem",IF(I22&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G22" s="42" t="str">
+      <c r="G22" s="43" t="str">
         <f aca="false">IF(B22="","",B22/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H22" s="42" t="str">
+      <c r="H22" s="43" t="str">
         <f aca="false">IF(B22="","",G22+C22)</f>
         <v/>
       </c>
-      <c r="I22" s="43" t="str">
+      <c r="I22" s="44" t="str">
         <f aca="false">IF(OR(B22="",D22=""),"",D22*(1-'Meu custo por hora'!$B$28)-H22)</f>
         <v/>
       </c>
       <c r="J22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40" t="str">
+      <c r="A23" s="38"/>
+      <c r="B23" s="39"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="41" t="str">
         <f aca="false">IF(B23="","",ROUNDUP(H23/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F23" s="41" t="str">
+      <c r="F23" s="42" t="str">
         <f aca="false">IF(OR(B23="",D23=""),"",IF(D23&gt;=E23,"OK: cobre custos e margem",IF(I23&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G23" s="42" t="str">
+      <c r="G23" s="43" t="str">
         <f aca="false">IF(B23="","",B23/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H23" s="42" t="str">
+      <c r="H23" s="43" t="str">
         <f aca="false">IF(B23="","",G23+C23)</f>
         <v/>
       </c>
-      <c r="I23" s="43" t="str">
+      <c r="I23" s="44" t="str">
         <f aca="false">IF(OR(B23="",D23=""),"",D23*(1-'Meu custo por hora'!$B$28)-H23)</f>
         <v/>
       </c>
       <c r="J23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="40" t="str">
+      <c r="A24" s="38"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="41" t="str">
         <f aca="false">IF(B24="","",ROUNDUP(H24/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F24" s="41" t="str">
+      <c r="F24" s="42" t="str">
         <f aca="false">IF(OR(B24="",D24=""),"",IF(D24&gt;=E24,"OK: cobre custos e margem",IF(I24&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G24" s="42" t="str">
+      <c r="G24" s="43" t="str">
         <f aca="false">IF(B24="","",B24/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H24" s="42" t="str">
+      <c r="H24" s="43" t="str">
         <f aca="false">IF(B24="","",G24+C24)</f>
         <v/>
       </c>
-      <c r="I24" s="43" t="str">
+      <c r="I24" s="44" t="str">
         <f aca="false">IF(OR(B24="",D24=""),"",D24*(1-'Meu custo por hora'!$B$28)-H24)</f>
         <v/>
       </c>
       <c r="J24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="39"/>
-      <c r="E25" s="40" t="str">
+      <c r="A25" s="38"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="41" t="str">
         <f aca="false">IF(B25="","",ROUNDUP(H25/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F25" s="41" t="str">
+      <c r="F25" s="42" t="str">
         <f aca="false">IF(OR(B25="",D25=""),"",IF(D25&gt;=E25,"OK: cobre custos e margem",IF(I25&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G25" s="42" t="str">
+      <c r="G25" s="43" t="str">
         <f aca="false">IF(B25="","",B25/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H25" s="42" t="str">
+      <c r="H25" s="43" t="str">
         <f aca="false">IF(B25="","",G25+C25)</f>
         <v/>
       </c>
-      <c r="I25" s="43" t="str">
+      <c r="I25" s="44" t="str">
         <f aca="false">IF(OR(B25="",D25=""),"",D25*(1-'Meu custo por hora'!$B$28)-H25)</f>
         <v/>
       </c>
       <c r="J25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="37"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="40" t="str">
+      <c r="A26" s="38"/>
+      <c r="B26" s="39"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="41" t="str">
         <f aca="false">IF(B26="","",ROUNDUP(H26/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F26" s="41" t="str">
+      <c r="F26" s="42" t="str">
         <f aca="false">IF(OR(B26="",D26=""),"",IF(D26&gt;=E26,"OK: cobre custos e margem",IF(I26&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G26" s="42" t="str">
+      <c r="G26" s="43" t="str">
         <f aca="false">IF(B26="","",B26/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H26" s="42" t="str">
+      <c r="H26" s="43" t="str">
         <f aca="false">IF(B26="","",G26+C26)</f>
         <v/>
       </c>
-      <c r="I26" s="43" t="str">
+      <c r="I26" s="44" t="str">
         <f aca="false">IF(OR(B26="",D26=""),"",D26*(1-'Meu custo por hora'!$B$28)-H26)</f>
         <v/>
       </c>
       <c r="J26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="37"/>
-      <c r="B27" s="38"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40" t="str">
+      <c r="A27" s="38"/>
+      <c r="B27" s="39"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="41" t="str">
         <f aca="false">IF(B27="","",ROUNDUP(H27/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F27" s="41" t="str">
+      <c r="F27" s="42" t="str">
         <f aca="false">IF(OR(B27="",D27=""),"",IF(D27&gt;=E27,"OK: cobre custos e margem",IF(I27&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G27" s="42" t="str">
+      <c r="G27" s="43" t="str">
         <f aca="false">IF(B27="","",B27/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H27" s="42" t="str">
+      <c r="H27" s="43" t="str">
         <f aca="false">IF(B27="","",G27+C27)</f>
         <v/>
       </c>
-      <c r="I27" s="43" t="str">
+      <c r="I27" s="44" t="str">
         <f aca="false">IF(OR(B27="",D27=""),"",D27*(1-'Meu custo por hora'!$B$28)-H27)</f>
         <v/>
       </c>
       <c r="J27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="37"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="40" t="str">
+      <c r="A28" s="38"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="41" t="str">
         <f aca="false">IF(B28="","",ROUNDUP(H28/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F28" s="41" t="str">
+      <c r="F28" s="42" t="str">
         <f aca="false">IF(OR(B28="",D28=""),"",IF(D28&gt;=E28,"OK: cobre custos e margem",IF(I28&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G28" s="42" t="str">
+      <c r="G28" s="43" t="str">
         <f aca="false">IF(B28="","",B28/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H28" s="42" t="str">
+      <c r="H28" s="43" t="str">
         <f aca="false">IF(B28="","",G28+C28)</f>
         <v/>
       </c>
-      <c r="I28" s="43" t="str">
+      <c r="I28" s="44" t="str">
         <f aca="false">IF(OR(B28="",D28=""),"",D28*(1-'Meu custo por hora'!$B$28)-H28)</f>
         <v/>
       </c>
       <c r="J28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="37"/>
-      <c r="B29" s="38"/>
-      <c r="C29" s="39"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="40" t="str">
+      <c r="A29" s="38"/>
+      <c r="B29" s="39"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="40"/>
+      <c r="E29" s="41" t="str">
         <f aca="false">IF(B29="","",ROUNDUP(H29/(1-'Meu custo por hora'!$B$28-'Meu custo por hora'!$B$29),0))</f>
         <v/>
       </c>
-      <c r="F29" s="41" t="str">
+      <c r="F29" s="42" t="str">
         <f aca="false">IF(OR(B29="",D29=""),"",IF(D29&gt;=E29,"OK: cobre custos e margem",IF(I29&gt;=0,"Atenção: pouca folga","PREJUÍZO: abaixo do custo")))</f>
         <v/>
       </c>
-      <c r="G29" s="42" t="str">
+      <c r="G29" s="43" t="str">
         <f aca="false">IF(B29="","",B29/60*'Meu custo por hora'!$B$25)</f>
         <v/>
       </c>
-      <c r="H29" s="42" t="str">
+      <c r="H29" s="43" t="str">
         <f aca="false">IF(B29="","",G29+C29)</f>
         <v/>
       </c>
-      <c r="I29" s="43" t="str">
+      <c r="I29" s="44" t="str">
         <f aca="false">IF(OR(B29="",D29=""),"",D29*(1-'Meu custo por hora'!$B$28)-H29)</f>
         <v/>
       </c>
@@ -3669,59 +3903,59 @@
       <c r="J30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="44" t="s">
-        <v>80</v>
-      </c>
-      <c r="B31" s="44"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="44"/>
-      <c r="F31" s="44"/>
-      <c r="G31" s="44"/>
-      <c r="H31" s="44"/>
-      <c r="I31" s="44"/>
+      <c r="A31" s="45" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31" s="45"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="45"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="45"/>
+      <c r="G31" s="45"/>
+      <c r="H31" s="45"/>
+      <c r="I31" s="45"/>
       <c r="J31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="B32" s="44"/>
-      <c r="C32" s="44"/>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
+      <c r="A32" s="45" t="s">
+        <v>83</v>
+      </c>
+      <c r="B32" s="45"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="45"/>
+      <c r="G32" s="45"/>
+      <c r="H32" s="45"/>
+      <c r="I32" s="45"/>
       <c r="J32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="44" t="s">
-        <v>82</v>
-      </c>
-      <c r="B33" s="44"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
-      <c r="I33" s="44"/>
+      <c r="A33" s="45" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33" s="45"/>
+      <c r="C33" s="45"/>
+      <c r="D33" s="45"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="45"/>
+      <c r="G33" s="45"/>
+      <c r="H33" s="45"/>
+      <c r="I33" s="45"/>
       <c r="J33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="44" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="44"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="44"/>
-      <c r="E34" s="44"/>
-      <c r="F34" s="44"/>
-      <c r="G34" s="44"/>
-      <c r="H34" s="44"/>
-      <c r="I34" s="44"/>
+      <c r="A34" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" s="45"/>
+      <c r="C34" s="45"/>
+      <c r="D34" s="45"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="45"/>
+      <c r="G34" s="45"/>
+      <c r="H34" s="45"/>
+      <c r="I34" s="45"/>
       <c r="J34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3761,8 +3995,9 @@
       <c r="J37" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:J1"/>
+  <mergeCells count="8">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="G1:I1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A31:I31"/>
@@ -3781,16 +4016,23 @@
       <formula>LEFT($F5,4)="PREJ"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Digite o tempo em minutos (ex.: 45)." errorStyle="stop" errorTitle="Tempo em minutos" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B29" type="decimal">
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="lessThanOrEqual" prompt="Escreva o nome do serviço. Depois preencha tempo, material e quanto cobra hoje." promptTitle="Nome do serviço" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="A5:A29" type="textLength">
+      <formula1>60</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Digite o tempo em minutos (ex.: 45)." errorStyle="stop" errorTitle="Tempo em minutos" operator="between" prompt="Quantos minutos dura este atendimento (ex.: 45)." promptTitle="Tempo do serviço" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B5:B29" type="decimal">
       <formula1>1</formula1>
       <formula2>720</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Digite um valor em reais (ex.: 35)." errorStyle="stop" errorTitle="Valor em reais" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C5:D29" type="decimal">
+    <dataValidation allowBlank="true" error="Digite um valor em reais (ex.: 35)." errorStyle="stop" errorTitle="Valor em reais" operator="greaterThanOrEqual" prompt="Material: quanto você gasta em produtos neste atendimento. Cobro hoje: o preço que você cobra atualmente." promptTitle="Em reais" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C5:D29" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="G1" location="'Meu Painel'!A1" display="Próximo: Meu Painel  →"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3798,6 +4040,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3807,7 +4050,7 @@
     <tabColor rgb="FF5A1236"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -3815,9 +4058,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="3"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -3828,14 +4071,16 @@
       <c r="H1" s="19"/>
       <c r="I1" s="19"/>
       <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
+      <c r="K1" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -3885,81 +4130,81 @@
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6"/>
-      <c r="B5" s="45" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45" t="s">
-        <v>87</v>
-      </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45" t="s">
-        <v>88</v>
-      </c>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="45" t="s">
+      <c r="B5" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="L5" s="45"/>
-      <c r="M5" s="45"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46" t="s">
+        <v>91</v>
+      </c>
+      <c r="I5" s="46"/>
+      <c r="J5" s="46"/>
+      <c r="K5" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
       <c r="N5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
-      <c r="B6" s="46" t="n">
+      <c r="B6" s="47" t="n">
         <f aca="false">'Meu custo por hora'!B25</f>
         <v>35.6191152957897</v>
       </c>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="47" t="n">
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="48" t="n">
         <f aca="false">COUNT('Meus serviços'!B5:B29)</f>
         <v>8</v>
       </c>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47" t="n">
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48" t="n">
         <f aca="false">COUNTIF('Meus serviços'!F5:F29,"Atenção*")+COUNTIF('Meus serviços'!F5:F29,"PREJUÍZO*")</f>
         <v>2</v>
       </c>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="48" t="n">
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="49" t="n">
         <f aca="false">COUNTIF('Meus serviços'!F5:F29,"PREJUÍZO*")</f>
         <v>1</v>
       </c>
-      <c r="L6" s="48"/>
-      <c r="M6" s="48"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="49"/>
       <c r="N6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
-      <c r="B7" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49" t="s">
-        <v>91</v>
-      </c>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49" t="s">
-        <v>92</v>
-      </c>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49" t="s">
+      <c r="B7" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="L7" s="49"/>
-      <c r="M7" s="49"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="I7" s="50"/>
+      <c r="J7" s="50"/>
+      <c r="K7" s="50" t="s">
+        <v>96</v>
+      </c>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
       <c r="N7" s="6"/>
     </row>
-    <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -3975,60 +4220,83 @@
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
-      <c r="B9" s="50" t="str">
-        <f aca="false">IF(K6&gt;0,"Atenção: "&amp;K6&amp;" serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.",IF(H6&gt;0,"Alguns serviços têm pouca folga. Compare o preço de hoje com o preço sugerido.","Os preços cadastrados cobrem seus custos e a margem. Revise quando seus gastos mudarem."))</f>
-        <v>Atenção: 1 serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.</v>
-      </c>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="50"/>
+      <c r="B9" s="46" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="I9" s="46"/>
+      <c r="J9" s="46"/>
+      <c r="K9" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="L9" s="46"/>
+      <c r="M9" s="46"/>
       <c r="N9" s="6"/>
     </row>
-    <row r="10" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
+      <c r="B10" s="51" t="n">
+        <f aca="false">COUNTIF('Meus serviços'!F5:F29,"OK*")</f>
+        <v>6</v>
+      </c>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="52" t="n">
+        <f aca="false">IFERROR(AVERAGE('Meus serviços'!I5:I29),0)</f>
+        <v>30.9269171552081</v>
+      </c>
+      <c r="F10" s="52"/>
+      <c r="G10" s="52"/>
+      <c r="H10" s="53" t="str">
+        <f aca="false">IFERROR(INDEX('Meus serviços'!A5:A29,MATCH(MAX('Meus serviços'!I5:I29),'Meus serviços'!I5:I29,0)),"-")</f>
+        <v>Extensão de cílios</v>
+      </c>
+      <c r="I10" s="53"/>
+      <c r="J10" s="53"/>
+      <c r="K10" s="54" t="str">
+        <f aca="false">IFERROR(INDEX('Meus serviços'!A5:A29,MATCH(MIN('Meus serviços'!I5:I29),'Meus serviços'!I5:I29,0)),"-")</f>
+        <v>Manicure (mão)</v>
+      </c>
+      <c r="L10" s="54"/>
+      <c r="M10" s="54"/>
       <c r="N10" s="6"/>
     </row>
-    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
-      <c r="B11" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
+      <c r="B11" s="50" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="50"/>
+      <c r="D11" s="50"/>
+      <c r="E11" s="50" t="s">
+        <v>102</v>
+      </c>
+      <c r="F11" s="50"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="I11" s="50"/>
+      <c r="J11" s="50"/>
+      <c r="K11" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="L11" s="50"/>
+      <c r="M11" s="50"/>
       <c r="N11" s="6"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -4044,23 +4312,26 @@
       <c r="M12" s="6"/>
       <c r="N12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
+      <c r="B13" s="55" t="str">
+        <f aca="false">IF(K6&gt;0,"Atenção: "&amp;K6&amp;" serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.",IF(H6&gt;0,"Alguns serviços têm pouca folga. Compare o preço de hoje com o preço sugerido.","Os preços cadastrados cobrem seus custos e a margem. Revise quando seus gastos mudarem."))</f>
+        <v>Atenção: 1 serviço(s) estão com preço abaixo do custo. Veja o preço sugerido na aba Meus serviços.</v>
+      </c>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="55"/>
+      <c r="K13" s="55"/>
+      <c r="L13" s="55"/>
+      <c r="M13" s="55"/>
       <c r="N13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -4076,20 +4347,22 @@
       <c r="M14" s="6"/>
       <c r="N14" s="6"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
+      <c r="B15" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
       <c r="N15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4350,20 +4623,18 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6"/>
-      <c r="B32" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="C32" s="44"/>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44"/>
-      <c r="K32" s="44"/>
-      <c r="L32" s="44"/>
-      <c r="M32" s="44"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="6"/>
       <c r="N32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4416,23 +4687,122 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
+      <c r="B36" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="45"/>
+      <c r="D36" s="45"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="45"/>
+      <c r="G36" s="45"/>
+      <c r="H36" s="45"/>
+      <c r="I36" s="45"/>
+      <c r="J36" s="45"/>
+      <c r="K36" s="45"/>
+      <c r="L36" s="45"/>
+      <c r="M36" s="45"/>
       <c r="N36" s="6"/>
     </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6"/>
+      <c r="K38" s="6"/>
+      <c r="L38" s="6"/>
+      <c r="M38" s="6"/>
+      <c r="N38" s="6"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="6"/>
+      <c r="K39" s="6"/>
+      <c r="L39" s="6"/>
+      <c r="M39" s="6"/>
+      <c r="N39" s="6"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6"/>
+      <c r="K40" s="6"/>
+      <c r="L40" s="6"/>
+      <c r="M40" s="6"/>
+      <c r="N40" s="6"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="6"/>
+      <c r="L41" s="6"/>
+      <c r="M41" s="6"/>
+      <c r="N41" s="6"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6"/>
+      <c r="L42" s="6"/>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="31">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="K1:M1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="B5:D5"/>
@@ -4447,10 +4817,25 @@
     <mergeCell ref="E7:G7"/>
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="K7:M7"/>
-    <mergeCell ref="B9:M9"/>
-    <mergeCell ref="B11:M11"/>
-    <mergeCell ref="B32:M32"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="B13:M13"/>
+    <mergeCell ref="B15:M15"/>
+    <mergeCell ref="B36:M36"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K1" location="'Tabela para divulgar'!A1" display="Ver Tabela para divulgar  →"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4478,12 +4863,12 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="51" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
+      <c r="A1" s="56" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
     </row>
     <row r="2" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5"/>
@@ -4493,10 +4878,10 @@
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6"/>
-      <c r="B3" s="52" t="s">
-        <v>97</v>
-      </c>
-      <c r="C3" s="52"/>
+      <c r="B3" s="57" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="57"/>
       <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4507,21 +4892,21 @@
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6"/>
-      <c r="B5" s="53" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="54" t="s">
-        <v>98</v>
+      <c r="B5" s="58" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>109</v>
       </c>
       <c r="D5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
-      <c r="B6" s="55" t="str">
+      <c r="B6" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B5="","",'Meus serviços'!A5)</f>
         <v>Corte feminino</v>
       </c>
-      <c r="C6" s="56" t="n">
+      <c r="C6" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B5="","",IF('Meus serviços'!D5&gt;='Meus serviços'!E5,'Meus serviços'!D5,'Meus serviços'!E5))</f>
         <v>80</v>
       </c>
@@ -4529,11 +4914,11 @@
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6"/>
-      <c r="B7" s="55" t="str">
+      <c r="B7" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B6="","",'Meus serviços'!A6)</f>
         <v>Escova</v>
       </c>
-      <c r="C7" s="56" t="n">
+      <c r="C7" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B6="","",IF('Meus serviços'!D6&gt;='Meus serviços'!E6,'Meus serviços'!D6,'Meus serviços'!E6))</f>
         <v>39</v>
       </c>
@@ -4541,11 +4926,11 @@
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6"/>
-      <c r="B8" s="55" t="str">
+      <c r="B8" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B7="","",'Meus serviços'!A7)</f>
         <v>Manicure (mão)</v>
       </c>
-      <c r="C8" s="56" t="n">
+      <c r="C8" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B7="","",IF('Meus serviços'!D7&gt;='Meus serviços'!E7,'Meus serviços'!D7,'Meus serviços'!E7))</f>
         <v>36</v>
       </c>
@@ -4553,11 +4938,11 @@
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6"/>
-      <c r="B9" s="55" t="str">
+      <c r="B9" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B8="","",'Meus serviços'!A8)</f>
         <v>Design de sobrancelha</v>
       </c>
-      <c r="C9" s="56" t="n">
+      <c r="C9" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B8="","",IF('Meus serviços'!D8&gt;='Meus serviços'!E8,'Meus serviços'!D8,'Meus serviços'!E8))</f>
         <v>40</v>
       </c>
@@ -4565,11 +4950,11 @@
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6"/>
-      <c r="B10" s="55" t="str">
+      <c r="B10" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B9="","",'Meus serviços'!A9)</f>
         <v>Limpeza de pele</v>
       </c>
-      <c r="C10" s="56" t="n">
+      <c r="C10" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B9="","",IF('Meus serviços'!D9&gt;='Meus serviços'!E9,'Meus serviços'!D9,'Meus serviços'!E9))</f>
         <v>120</v>
       </c>
@@ -4577,11 +4962,11 @@
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
-      <c r="B11" s="55" t="str">
+      <c r="B11" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B10="","",'Meus serviços'!A10)</f>
         <v>Massagem relaxante</v>
       </c>
-      <c r="C11" s="56" t="n">
+      <c r="C11" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B10="","",IF('Meus serviços'!D10&gt;='Meus serviços'!E10,'Meus serviços'!D10,'Meus serviços'!E10))</f>
         <v>100</v>
       </c>
@@ -4589,11 +4974,11 @@
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6"/>
-      <c r="B12" s="55" t="str">
+      <c r="B12" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B11="","",'Meus serviços'!A11)</f>
         <v>Extensão de cílios</v>
       </c>
-      <c r="C12" s="56" t="n">
+      <c r="C12" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B11="","",IF('Meus serviços'!D11&gt;='Meus serviços'!E11,'Meus serviços'!D11,'Meus serviços'!E11))</f>
         <v>180</v>
       </c>
@@ -4601,11 +4986,11 @@
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6"/>
-      <c r="B13" s="55" t="str">
+      <c r="B13" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B12="","",'Meus serviços'!A12)</f>
         <v>Depilação (perna)</v>
       </c>
-      <c r="C13" s="56" t="n">
+      <c r="C13" s="61" t="n">
         <f aca="false">IF('Meus serviços'!B12="","",IF('Meus serviços'!D12&gt;='Meus serviços'!E12,'Meus serviços'!D12,'Meus serviços'!E12))</f>
         <v>55</v>
       </c>
@@ -4613,11 +4998,11 @@
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6"/>
-      <c r="B14" s="55" t="str">
+      <c r="B14" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B13="","",'Meus serviços'!A13)</f>
         <v/>
       </c>
-      <c r="C14" s="56" t="str">
+      <c r="C14" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B13="","",IF('Meus serviços'!D13&gt;='Meus serviços'!E13,'Meus serviços'!D13,'Meus serviços'!E13))</f>
         <v/>
       </c>
@@ -4625,11 +5010,11 @@
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6"/>
-      <c r="B15" s="55" t="str">
+      <c r="B15" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B14="","",'Meus serviços'!A14)</f>
         <v/>
       </c>
-      <c r="C15" s="56" t="str">
+      <c r="C15" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B14="","",IF('Meus serviços'!D14&gt;='Meus serviços'!E14,'Meus serviços'!D14,'Meus serviços'!E14))</f>
         <v/>
       </c>
@@ -4637,11 +5022,11 @@
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6"/>
-      <c r="B16" s="55" t="str">
+      <c r="B16" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B15="","",'Meus serviços'!A15)</f>
         <v/>
       </c>
-      <c r="C16" s="56" t="str">
+      <c r="C16" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B15="","",IF('Meus serviços'!D15&gt;='Meus serviços'!E15,'Meus serviços'!D15,'Meus serviços'!E15))</f>
         <v/>
       </c>
@@ -4649,11 +5034,11 @@
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
-      <c r="B17" s="55" t="str">
+      <c r="B17" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B16="","",'Meus serviços'!A16)</f>
         <v/>
       </c>
-      <c r="C17" s="56" t="str">
+      <c r="C17" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B16="","",IF('Meus serviços'!D16&gt;='Meus serviços'!E16,'Meus serviços'!D16,'Meus serviços'!E16))</f>
         <v/>
       </c>
@@ -4661,11 +5046,11 @@
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
-      <c r="B18" s="55" t="str">
+      <c r="B18" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B17="","",'Meus serviços'!A17)</f>
         <v/>
       </c>
-      <c r="C18" s="56" t="str">
+      <c r="C18" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B17="","",IF('Meus serviços'!D17&gt;='Meus serviços'!E17,'Meus serviços'!D17,'Meus serviços'!E17))</f>
         <v/>
       </c>
@@ -4673,11 +5058,11 @@
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6"/>
-      <c r="B19" s="55" t="str">
+      <c r="B19" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B18="","",'Meus serviços'!A18)</f>
         <v/>
       </c>
-      <c r="C19" s="56" t="str">
+      <c r="C19" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B18="","",IF('Meus serviços'!D18&gt;='Meus serviços'!E18,'Meus serviços'!D18,'Meus serviços'!E18))</f>
         <v/>
       </c>
@@ -4685,11 +5070,11 @@
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
-      <c r="B20" s="55" t="str">
+      <c r="B20" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B19="","",'Meus serviços'!A19)</f>
         <v/>
       </c>
-      <c r="C20" s="56" t="str">
+      <c r="C20" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B19="","",IF('Meus serviços'!D19&gt;='Meus serviços'!E19,'Meus serviços'!D19,'Meus serviços'!E19))</f>
         <v/>
       </c>
@@ -4697,11 +5082,11 @@
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6"/>
-      <c r="B21" s="55" t="str">
+      <c r="B21" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B20="","",'Meus serviços'!A20)</f>
         <v/>
       </c>
-      <c r="C21" s="56" t="str">
+      <c r="C21" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B20="","",IF('Meus serviços'!D20&gt;='Meus serviços'!E20,'Meus serviços'!D20,'Meus serviços'!E20))</f>
         <v/>
       </c>
@@ -4709,11 +5094,11 @@
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6"/>
-      <c r="B22" s="55" t="str">
+      <c r="B22" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B21="","",'Meus serviços'!A21)</f>
         <v/>
       </c>
-      <c r="C22" s="56" t="str">
+      <c r="C22" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B21="","",IF('Meus serviços'!D21&gt;='Meus serviços'!E21,'Meus serviços'!D21,'Meus serviços'!E21))</f>
         <v/>
       </c>
@@ -4721,11 +5106,11 @@
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6"/>
-      <c r="B23" s="55" t="str">
+      <c r="B23" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B22="","",'Meus serviços'!A22)</f>
         <v/>
       </c>
-      <c r="C23" s="56" t="str">
+      <c r="C23" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B22="","",IF('Meus serviços'!D22&gt;='Meus serviços'!E22,'Meus serviços'!D22,'Meus serviços'!E22))</f>
         <v/>
       </c>
@@ -4733,11 +5118,11 @@
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6"/>
-      <c r="B24" s="55" t="str">
+      <c r="B24" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B23="","",'Meus serviços'!A23)</f>
         <v/>
       </c>
-      <c r="C24" s="56" t="str">
+      <c r="C24" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B23="","",IF('Meus serviços'!D23&gt;='Meus serviços'!E23,'Meus serviços'!D23,'Meus serviços'!E23))</f>
         <v/>
       </c>
@@ -4745,11 +5130,11 @@
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6"/>
-      <c r="B25" s="55" t="str">
+      <c r="B25" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B24="","",'Meus serviços'!A24)</f>
         <v/>
       </c>
-      <c r="C25" s="56" t="str">
+      <c r="C25" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B24="","",IF('Meus serviços'!D24&gt;='Meus serviços'!E24,'Meus serviços'!D24,'Meus serviços'!E24))</f>
         <v/>
       </c>
@@ -4757,11 +5142,11 @@
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6"/>
-      <c r="B26" s="55" t="str">
+      <c r="B26" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B25="","",'Meus serviços'!A25)</f>
         <v/>
       </c>
-      <c r="C26" s="56" t="str">
+      <c r="C26" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B25="","",IF('Meus serviços'!D25&gt;='Meus serviços'!E25,'Meus serviços'!D25,'Meus serviços'!E25))</f>
         <v/>
       </c>
@@ -4769,11 +5154,11 @@
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6"/>
-      <c r="B27" s="55" t="str">
+      <c r="B27" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B26="","",'Meus serviços'!A26)</f>
         <v/>
       </c>
-      <c r="C27" s="56" t="str">
+      <c r="C27" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B26="","",IF('Meus serviços'!D26&gt;='Meus serviços'!E26,'Meus serviços'!D26,'Meus serviços'!E26))</f>
         <v/>
       </c>
@@ -4781,11 +5166,11 @@
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6"/>
-      <c r="B28" s="55" t="str">
+      <c r="B28" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B27="","",'Meus serviços'!A27)</f>
         <v/>
       </c>
-      <c r="C28" s="56" t="str">
+      <c r="C28" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B27="","",IF('Meus serviços'!D27&gt;='Meus serviços'!E27,'Meus serviços'!D27,'Meus serviços'!E27))</f>
         <v/>
       </c>
@@ -4793,11 +5178,11 @@
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6"/>
-      <c r="B29" s="55" t="str">
+      <c r="B29" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B28="","",'Meus serviços'!A28)</f>
         <v/>
       </c>
-      <c r="C29" s="56" t="str">
+      <c r="C29" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B28="","",IF('Meus serviços'!D28&gt;='Meus serviços'!E28,'Meus serviços'!D28,'Meus serviços'!E28))</f>
         <v/>
       </c>
@@ -4805,11 +5190,11 @@
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6"/>
-      <c r="B30" s="55" t="str">
+      <c r="B30" s="60" t="str">
         <f aca="false">IF('Meus serviços'!B29="","",'Meus serviços'!A29)</f>
         <v/>
       </c>
-      <c r="C30" s="56" t="str">
+      <c r="C30" s="61" t="str">
         <f aca="false">IF('Meus serviços'!B29="","",IF('Meus serviços'!D29&gt;='Meus serviços'!E29,'Meus serviços'!D29,'Meus serviços'!E29))</f>
         <v/>
       </c>
@@ -4831,10 +5216,10 @@
     </row>
     <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6"/>
-      <c r="B33" s="57" t="s">
-        <v>99</v>
-      </c>
-      <c r="C33" s="57"/>
+      <c r="B33" s="62" t="s">
+        <v>110</v>
+      </c>
+      <c r="C33" s="62"/>
       <c r="D33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Resultado da planilha em rosa (distinto do amarelo de preenchimento), no site e no Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VVXSWQenri3WwETC67snQx
</commit_message>
<xml_diff>
--- a/Calculadora-Preco-Certo.xlsx
+++ b/Calculadora-Preco-Certo.xlsx
@@ -89,7 +89,7 @@
     <t xml:space="preserve">Resultado</t>
   </si>
   <si>
-    <t xml:space="preserve">Preço sugerido e resultados principais.</t>
+    <t xml:space="preserve">Preço sugerido e resultados principais, calculados sozinhos.</t>
   </si>
   <si>
     <t xml:space="preserve">Importante</t>
@@ -660,7 +660,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -711,6 +711,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFDCEB"/>
+        <bgColor rgb="FFFDE0E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFCE9F0"/>
         <bgColor rgb="FFF8EDE6"/>
       </patternFill>
@@ -734,7 +740,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="16">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -782,6 +788,21 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFE91E78"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE91E78"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE91E78"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE91E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -797,6 +818,21 @@
         <color rgb="FFE0B84C"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FFE91E78"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE91E78"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE91E78"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE91E78"/>
+      </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -996,15 +1032,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1012,15 +1048,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="7" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1032,11 +1068,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="11" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="12" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="11" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="19" fillId="12" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1052,63 +1088,63 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="23" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="23" fillId="6" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="24" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="7" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="13" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="8" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="20" fillId="8" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="8" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="20" fillId="8" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="7" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="27" fillId="9" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="20" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="20" fillId="6" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="20" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1116,43 +1152,43 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="6" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="29" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="29" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="29" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="29" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="30" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="30" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="6" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="31" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="31" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="32" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="32" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="33" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="33" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="34" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="34" fillId="6" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="11" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="12" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1164,11 +1200,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1271,7 +1307,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFF0D5DF"/>
       <rgbColor rgb="FF878787"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FFFFDCEB"/>
       <rgbColor rgb="FFC2185B"/>
       <rgbColor rgb="FFFFF3C4"/>
       <rgbColor rgb="FFE3F4E7"/>
@@ -1575,11 +1611,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="25424270"/>
-        <c:axId val="80355751"/>
+        <c:axId val="5119810"/>
+        <c:axId val="70011417"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25424270"/>
+        <c:axId val="5119810"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1611,7 +1647,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80355751"/>
+        <c:crossAx val="70011417"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1619,7 +1655,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80355751"/>
+        <c:axId val="70011417"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1661,7 +1697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25424270"/>
+        <c:crossAx val="5119810"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>